<commit_message>
Add Oradea, Lugoj and Cenei battles
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/conflicte_militare/conflicte_militare_romania.xlsx
+++ b/data/conflicte_militare/conflicte_militare_romania.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Dicționar" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conflicte'!$A$1:$U$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Conflicte'!$A$1:$U$202</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U199"/>
+  <dimension ref="A1:U202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14956,7 +14956,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>Șoplea (județul Mureș)</t>
+          <t>Șoplea (comuna Drăgănești, județul Prahova)</t>
         </is>
       </c>
       <c r="K153" s="2" t="n">
@@ -14964,19 +14964,19 @@
       </c>
       <c r="L153" s="2" t="inlineStr">
         <is>
-          <t>Mureș</t>
+          <t>Prahova</t>
         </is>
       </c>
       <c r="M153" s="2" t="inlineStr">
         <is>
-          <t>Transilvania</t>
+          <t>Țara Românească</t>
         </is>
       </c>
       <c r="N153" s="2" t="n">
-        <v>46.45</v>
+        <v>44.828</v>
       </c>
       <c r="O153" s="2" t="n">
-        <v>24.4</v>
+        <v>26.288</v>
       </c>
       <c r="P153" s="2" t="inlineStr">
         <is>
@@ -15397,75 +15397,75 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Războiul Ruso-Turc (1710–1711) și Bătălia de la Stănilești</t>
+          <t>Asediul Oradiei (1692)</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Război / bătălie</t>
+          <t>Asediu</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>1710</t>
+          <t>1692</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>1711</t>
+          <t>1692</t>
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>1710</v>
+        <v>1692</v>
       </c>
       <c r="G158" s="2" t="n">
-        <v>1711</v>
+        <v>1692</v>
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>sec. XVIII d.Hr.</t>
+          <t>sec. XVII d.Hr.</t>
         </is>
       </c>
       <c r="I158" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>Stănilești, pe Prut (județul Vaslui)</t>
+          <t>Oradea (județul Bihor)</t>
         </is>
       </c>
       <c r="K158" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>Vaslui</t>
+          <t>Bihor</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Crișana</t>
         </is>
       </c>
       <c r="N158" s="2" t="n">
-        <v>46.63</v>
+        <v>47.05</v>
       </c>
       <c r="O158" s="2" t="n">
-        <v>28.14</v>
+        <v>21.93</v>
       </c>
       <c r="P158" s="2" t="inlineStr">
         <is>
-          <t>Rusia (Petru cel Mare) și Moldova (Dimitrie Cantemir) vs. Imperiul Otoman și tătari</t>
+          <t>Imperiul Habsburgic vs. Imperiul Otoman (garnizoana Cetății Oradea)</t>
         </is>
       </c>
       <c r="Q158" s="2" t="inlineStr">
         <is>
-          <t>Domnitorul Moldovei, Dimitrie Cantemir, se aliază secret cu țarul Petru cel Mare (Tratatul de la Luțk), încercând să elibereze țara de suzeranitatea otomană. La Stănilești, pe Prut (iulie 1711), armatele moldo-ruse sunt încercuite și înfrânte de otomani. Cantemir se exilează în Rusia, iar Poarta introduce regimul fanariot în Moldova (1711) și apoi în Țara Românească (1716).</t>
+          <t>În timpul Marelui Război Turcesc, armata habsburgică asediază Cetatea Oradea, important centru al stăpânirii otomane din Crișana. După blocarea și bombardarea fortificației, garnizoana otomană capitulează, iar orașul intră sub control habsburgic.</t>
         </is>
       </c>
       <c r="R158" s="2" t="inlineStr">
         <is>
-          <t>Înfrângerea moldo-rusă; introducerea regimului fanariot</t>
+          <t>Victorie habsburgică și ocuparea Oradiei</t>
         </is>
       </c>
       <c r="S158" s="2" t="inlineStr">
@@ -15480,7 +15480,7 @@
       </c>
       <c r="U158" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XVIII d.Hr., pct. 1</t>
+          <t>Completare solicitată — Marele Război Turcesc</t>
         </is>
       </c>
     </row>
@@ -15492,90 +15492,90 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Războiul Austro-Turc (1716–1718)</t>
+          <t>Bătălia de la Lugoj (1695)</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Război</t>
+          <t>Bătălie</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>1716</t>
+          <t>1695</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>1718</t>
+          <t>1695</t>
         </is>
       </c>
       <c r="F159" s="2" t="n">
-        <v>1716</v>
+        <v>1695</v>
       </c>
       <c r="G159" s="2" t="n">
-        <v>1718</v>
+        <v>1695</v>
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>sec. XVIII d.Hr.</t>
+          <t>sec. XVII d.Hr.</t>
         </is>
       </c>
       <c r="I159" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J159" s="2" t="inlineStr">
         <is>
-          <t>Banat și Țara Românească</t>
+          <t>Lugoj (județul Timiș)</t>
         </is>
       </c>
       <c r="K159" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L159" s="2" t="inlineStr">
         <is>
+          <t>Timiș</t>
+        </is>
+      </c>
+      <c r="M159" s="2" t="inlineStr">
+        <is>
+          <t>Banat</t>
+        </is>
+      </c>
+      <c r="N159" s="2" t="n">
+        <v>45.69</v>
+      </c>
+      <c r="O159" s="2" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="P159" s="2" t="inlineStr">
+        <is>
+          <t>Imperiul Otoman vs. Imperiul Habsburgic</t>
+        </is>
+      </c>
+      <c r="Q159" s="2" t="inlineStr">
+        <is>
+          <t>În cadrul Marelui Război Turcesc, armata otomană condusă de sultanul Mustafa al II-lea înfruntă forțele habsburgice din Banat în apropierea Lugojului. Trupele imperiale sunt învinse, iar comandantul lor, feldmareșalul Friedrich von Veterani, este ucis în timpul retragerii.</t>
+        </is>
+      </c>
+      <c r="R159" s="2" t="inlineStr">
+        <is>
+          <t>Victorie otomană</t>
+        </is>
+      </c>
+      <c r="S159" s="2" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
+      <c r="T159" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M159" s="2" t="inlineStr">
-        <is>
-          <t>Banat / Țara Românească</t>
-        </is>
-      </c>
-      <c r="N159" s="2" t="n">
-        <v>45.5</v>
-      </c>
-      <c r="O159" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="P159" s="2" t="inlineStr">
-        <is>
-          <t>Imperiul Habsburgic vs. Imperiul Otoman</t>
-        </is>
-      </c>
-      <c r="Q159" s="2" t="inlineStr">
-        <is>
-          <t>Trupele habsburgice atacă fortărețele otomane și pătrund adânc în Banat și Țara Românească. Conflictul se încheie prin Pacea de la Passarowitz (1718), prin care Imperiul Habsburgic anexează Banatul și Oltenia (aceasta fiind retrocedată Țării Românești două decenii mai târziu).</t>
-        </is>
-      </c>
-      <c r="R159" s="2" t="inlineStr">
-        <is>
-          <t>Anexarea Banatului și Olteniei de către Habsburgi</t>
-        </is>
-      </c>
-      <c r="S159" s="2" t="inlineStr">
-        <is>
-          <t>Da</t>
-        </is>
-      </c>
-      <c r="T159" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="U159" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XVIII d.Hr., pct. 2</t>
+          <t>Completare solicitată — Marele Război Turcesc</t>
         </is>
       </c>
     </row>
@@ -15587,90 +15587,90 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Războiul Ruso-Austro-Turc (1735–1739)</t>
+          <t>Bătălia de la Cenei (1696)</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Război</t>
+          <t>Bătălie</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>1735</t>
+          <t>1696</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>1739</t>
+          <t>1696</t>
         </is>
       </c>
       <c r="F160" s="2" t="n">
-        <v>1735</v>
+        <v>1696</v>
       </c>
       <c r="G160" s="2" t="n">
-        <v>1739</v>
+        <v>1696</v>
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>sec. XVIII d.Hr.</t>
+          <t>sec. XVII d.Hr.</t>
         </is>
       </c>
       <c r="I160" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J160" s="2" t="inlineStr">
         <is>
-          <t>Moldova (Iași), Oltenia și Muntenia</t>
+          <t>Cenei (județul Timiș)</t>
         </is>
       </c>
       <c r="K160" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L160" s="2" t="inlineStr">
         <is>
+          <t>Timiș</t>
+        </is>
+      </c>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>Banat</t>
+        </is>
+      </c>
+      <c r="N160" s="2" t="n">
+        <v>45.72</v>
+      </c>
+      <c r="O160" s="2" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="P160" s="2" t="inlineStr">
+        <is>
+          <t>Imperiul Habsburgic vs. Imperiul Otoman</t>
+        </is>
+      </c>
+      <c r="Q160" s="2" t="inlineStr">
+        <is>
+          <t>Armata habsburgică și cea otomană se confruntă lângă Cenei, în Banat, în continuarea operațiunilor Marelui Război Turcesc. Forțele habsburgice obțin victoria și își consolidează ofensiva împotriva pozițiilor otomane din regiune.</t>
+        </is>
+      </c>
+      <c r="R160" s="2" t="inlineStr">
+        <is>
+          <t>Victorie habsburgică</t>
+        </is>
+      </c>
+      <c r="S160" s="2" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
+      <c r="T160" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M160" s="2" t="inlineStr">
-        <is>
-          <t>Moldova / Oltenia / Muntenia</t>
-        </is>
-      </c>
-      <c r="N160" s="2" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="O160" s="2" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="P160" s="2" t="inlineStr">
-        <is>
-          <t>Rusia și Imperiul Habsburgic vs. Imperiul Otoman</t>
-        </is>
-      </c>
-      <c r="Q160" s="2" t="inlineStr">
-        <is>
-          <t>Teritoriul Moldovei și al Țării Românești este din nou teatru de război: trupele rusești ocupă Iașiul, iar austriecii luptă pe teritoriul Olteniei și în Muntenia. Se încheie prin Pacea de la Belgrad (1739), prin care Austria pierde Oltenia, care revine sub stăpânirea domniei de la București (și indirect sub suzeranitate otomană).</t>
-        </is>
-      </c>
-      <c r="R160" s="2" t="inlineStr">
-        <is>
-          <t>Revenirea Olteniei sub autoritatea Bucureștiului</t>
-        </is>
-      </c>
-      <c r="S160" s="2" t="inlineStr">
-        <is>
-          <t>Da</t>
-        </is>
-      </c>
-      <c r="T160" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="U160" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XVIII d.Hr., pct. 3</t>
+          <t>Completare solicitată — Marele Război Turcesc</t>
         </is>
       </c>
     </row>
@@ -15682,29 +15682,29 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Războiul Ruso-Turc (1768–1774) și ocupația Principatelor</t>
+          <t>Războiul Ruso-Turc (1710–1711) și Bătălia de la Stănilești</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Război / ocupație</t>
+          <t>Război / bătălie</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>1768</t>
+          <t>1710</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>1774</t>
+          <t>1711</t>
         </is>
       </c>
       <c r="F161" s="2" t="n">
-        <v>1768</v>
+        <v>1710</v>
       </c>
       <c r="G161" s="2" t="n">
-        <v>1774</v>
+        <v>1711</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
@@ -15716,7 +15716,7 @@
       </c>
       <c r="J161" s="2" t="inlineStr">
         <is>
-          <t>Moldova și Țara Românească (Bătăliile de la Larga și Cahul — azi Republica Moldova)</t>
+          <t>Stănilești, pe Prut (județul Vaslui)</t>
         </is>
       </c>
       <c r="K161" s="2" t="n">
@@ -15724,48 +15724,48 @@
       </c>
       <c r="L161" s="2" t="inlineStr">
         <is>
+          <t>Vaslui</t>
+        </is>
+      </c>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>Moldova</t>
+        </is>
+      </c>
+      <c r="N161" s="2" t="n">
+        <v>46.63</v>
+      </c>
+      <c r="O161" s="2" t="n">
+        <v>28.14</v>
+      </c>
+      <c r="P161" s="2" t="inlineStr">
+        <is>
+          <t>Rusia (Petru cel Mare) și Moldova (Dimitrie Cantemir) vs. Imperiul Otoman și tătari</t>
+        </is>
+      </c>
+      <c r="Q161" s="2" t="inlineStr">
+        <is>
+          <t>Domnitorul Moldovei, Dimitrie Cantemir, se aliază secret cu țarul Petru cel Mare (Tratatul de la Luțk), încercând să elibereze țara de suzeranitatea otomană. La Stănilești, pe Prut (iulie 1711), armatele moldo-ruse sunt încercuite și înfrânte de otomani. Cantemir se exilează în Rusia, iar Poarta introduce regimul fanariot în Moldova (1711) și apoi în Țara Românească (1716).</t>
+        </is>
+      </c>
+      <c r="R161" s="2" t="inlineStr">
+        <is>
+          <t>Înfrângerea moldo-rusă; introducerea regimului fanariot</t>
+        </is>
+      </c>
+      <c r="S161" s="2" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
+      <c r="T161" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M161" s="2" t="inlineStr">
-        <is>
-          <t>Moldova / Țara Românească</t>
-        </is>
-      </c>
-      <c r="N161" s="2" t="n">
-        <v>46.3</v>
-      </c>
-      <c r="O161" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="P161" s="2" t="inlineStr">
-        <is>
-          <t>Imperiul Rus vs. Imperiul Otoman</t>
-        </is>
-      </c>
-      <c r="Q161" s="2" t="inlineStr">
-        <is>
-          <t>Unul dintre cele mai distructive conflicte ale secolului pentru spațiul românesc: Moldova și Țara Românească sunt complet ocupate de armatele țariste, iar bătăliile importante de la Larga și Cahul se dau pe teritoriul basarabean de atunci. Pacea de la Kuciuk-Kainargi (1774) retrocedează formal Principatele otomanilor, dar Rusia obține dreptul de a interveni în protejarea creștinilor; în 1775 Austria anexează nordul Moldovei (Bucovina).</t>
-        </is>
-      </c>
-      <c r="R161" s="2" t="inlineStr">
-        <is>
-          <t>Ocupație și distrugeri; dreptul rusesc de intervenție; anexarea Bucovinei</t>
-        </is>
-      </c>
-      <c r="S161" s="2" t="inlineStr">
-        <is>
-          <t>Da</t>
-        </is>
-      </c>
-      <c r="T161" s="2" t="inlineStr">
-        <is>
-          <t>Bătăliile de la Larga și Cahul au avut loc în afara granițelor actuale ale României.</t>
-        </is>
-      </c>
       <c r="U161" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XVIII d.Hr., pct. 4</t>
+          <t>batalii.csv — sec. XVIII d.Hr., pct. 1</t>
         </is>
       </c>
     </row>
@@ -15777,29 +15777,29 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Războiul Ruso-Austro-Turc (1787–1792) și bătăliile de la Focșani și Râmnicu Sărat</t>
+          <t>Războiul Austro-Turc (1716–1718)</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Război / bătălii</t>
+          <t>Război</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>1787</t>
+          <t>1716</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>1792</t>
+          <t>1718</t>
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>1787</v>
+        <v>1716</v>
       </c>
       <c r="G162" s="2" t="n">
-        <v>1792</v>
+        <v>1718</v>
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
@@ -15811,7 +15811,7 @@
       </c>
       <c r="J162" s="2" t="inlineStr">
         <is>
-          <t>București, Iași, Focșani, Râmnicu Sărat</t>
+          <t>Banat și Țara Românească</t>
         </is>
       </c>
       <c r="K162" s="2" t="n">
@@ -15819,33 +15819,33 @@
       </c>
       <c r="L162" s="2" t="inlineStr">
         <is>
-          <t>Ilfov / Iași / Vrancea / Buzău</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M162" s="2" t="inlineStr">
         <is>
-          <t>Țara Românească / Moldova</t>
+          <t>Banat / Țara Românească</t>
         </is>
       </c>
       <c r="N162" s="2" t="n">
         <v>45.5</v>
       </c>
       <c r="O162" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="P162" s="2" t="inlineStr">
         <is>
-          <t>Rusia și Imperiul Habsburgic vs. Imperiul Otoman</t>
+          <t>Imperiul Habsburgic vs. Imperiul Otoman</t>
         </is>
       </c>
       <c r="Q162" s="2" t="inlineStr">
         <is>
-          <t>Alianța austro-rusă atacă Imperiul Otoman pe pământ românesc: Bucureștiul și Iașiul sunt ocupate militar de trupele aliate, iar generalul rus Suvorov obține victorii răsunătoare la Focșani (1789) și Râmnicu Sărat (1789). Războiul se încheie prin Pacea de la Șiștov (1791) cu Austria și Pacea de la Iași (1792) cu Rusia, când granița rusă ajunge pentru prima dată pe Nistru.</t>
+          <t>Trupele habsburgice atacă fortărețele otomane și pătrund adânc în Banat și Țara Românească. Conflictul se încheie prin Pacea de la Passarowitz (1718), prin care Imperiul Habsburgic anexează Banatul și Oltenia (aceasta fiind retrocedată Țării Românești două decenii mai târziu).</t>
         </is>
       </c>
       <c r="R162" s="2" t="inlineStr">
         <is>
-          <t>Ocupație militară; granița rusă pe Nistru; restabilirea suzeranității otomane</t>
+          <t>Anexarea Banatului și Olteniei de către Habsburgi</t>
         </is>
       </c>
       <c r="S162" s="2" t="inlineStr">
@@ -15860,7 +15860,7 @@
       </c>
       <c r="U162" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XVIII d.Hr., pct. 5</t>
+          <t>batalii.csv — sec. XVIII d.Hr., pct. 2</t>
         </is>
       </c>
     </row>
@@ -15872,7 +15872,7 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Războiul Ruso-Turc (1806–1812) și anexarea Basarabiei</t>
+          <t>Războiul Ruso-Austro-Turc (1735–1739)</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
@@ -15882,31 +15882,31 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>1806</t>
+          <t>1735</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>1812</t>
+          <t>1739</t>
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>1806</v>
+        <v>1735</v>
       </c>
       <c r="G163" s="2" t="n">
-        <v>1812</v>
+        <v>1739</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
-          <t>sec. XIX d.Hr.</t>
+          <t>sec. XVIII d.Hr.</t>
         </is>
       </c>
       <c r="I163" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J163" s="2" t="inlineStr">
         <is>
-          <t>Moldova (dintre Prut și Nistru) și Țara Românească</t>
+          <t>Moldova (Iași), Oltenia și Muntenia</t>
         </is>
       </c>
       <c r="K163" s="2" t="n">
@@ -15919,28 +15919,28 @@
       </c>
       <c r="M163" s="2" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Moldova / Oltenia / Muntenia</t>
         </is>
       </c>
       <c r="N163" s="2" t="n">
-        <v>47</v>
+        <v>46.7</v>
       </c>
       <c r="O163" s="2" t="n">
-        <v>28</v>
+        <v>26.5</v>
       </c>
       <c r="P163" s="2" t="inlineStr">
         <is>
-          <t>Imperiul Rus vs. Imperiul Otoman (principatele române ca teatru de război)</t>
+          <t>Rusia și Imperiul Habsburgic vs. Imperiul Otoman</t>
         </is>
       </c>
       <c r="Q163" s="2" t="inlineStr">
         <is>
-          <t>Spațiul românesc este teatru de operațiuni sau ocupat militar: războiul se încheie cu Pacea de la București, prin care Imperiul Rus anexează jumătatea de est a Moldovei — teritoriul dintre Prut și Nistru, numit ulterior Basarabia.</t>
+          <t>Teritoriul Moldovei și al Țării Românești este din nou teatru de război: trupele rusești ocupă Iașiul, iar austriecii luptă pe teritoriul Olteniei și în Muntenia. Se încheie prin Pacea de la Belgrad (1739), prin care Austria pierde Oltenia, care revine sub stăpânirea domniei de la București (și indirect sub suzeranitate otomană).</t>
         </is>
       </c>
       <c r="R163" s="2" t="inlineStr">
         <is>
-          <t>Anexarea Basarabiei de către Imperiul Rus</t>
+          <t>Revenirea Olteniei sub autoritatea Bucureștiului</t>
         </is>
       </c>
       <c r="S163" s="2" t="inlineStr">
@@ -15950,12 +15950,12 @@
       </c>
       <c r="T163" s="2" t="inlineStr">
         <is>
-          <t>Moștenirea teritorială a evenimentului privește și Republica Moldova de azi.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U163" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XIX d.Hr.</t>
+          <t>batalii.csv — sec. XVIII d.Hr., pct. 3</t>
         </is>
       </c>
     </row>
@@ -15967,41 +15967,41 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Revoluția lui Tudor Vladimirescu (1821)</t>
+          <t>Războiul Ruso-Turc (1768–1774) și ocupația Principatelor</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Revoltă / război intern</t>
+          <t>Război / ocupație</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1768</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>1821</t>
+          <t>1774</t>
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>1821</v>
+        <v>1768</v>
       </c>
       <c r="G164" s="2" t="n">
-        <v>1821</v>
+        <v>1774</v>
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>sec. XIX d.Hr.</t>
+          <t>sec. XVIII d.Hr.</t>
         </is>
       </c>
       <c r="I164" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J164" s="2" t="inlineStr">
         <is>
-          <t>Țara Românească: Gorj, Oltenia, București</t>
+          <t>Moldova și Țara Românească (Bătăliile de la Larga și Cahul — azi Republica Moldova)</t>
         </is>
       </c>
       <c r="K164" s="2" t="n">
@@ -16009,33 +16009,33 @@
       </c>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>Gorj / Dolj / Ilfov</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M164" s="2" t="inlineStr">
         <is>
-          <t>Țara Românească</t>
+          <t>Moldova / Țara Românească</t>
         </is>
       </c>
       <c r="N164" s="2" t="n">
-        <v>44.8</v>
+        <v>46.3</v>
       </c>
       <c r="O164" s="2" t="n">
-        <v>23.5</v>
+        <v>28</v>
       </c>
       <c r="P164" s="2" t="inlineStr">
         <is>
-          <t>Pandurii lui Tudor Vladimirescu și eteriștii (Alexandru Ipsilanti) vs. Imperiul Otoman</t>
+          <t>Imperiul Rus vs. Imperiul Otoman</t>
         </is>
       </c>
       <c r="Q164" s="2" t="inlineStr">
         <is>
-          <t>Mișcare socială și națională puternică în Țara Românească: se dau lupte între pandurii lui Tudor Vladimirescu, eteriștii (revoluționarii greci conduși de Alexandru Ipsilanti, care acționau tot pe teritoriu românesc) și armatele otomane venite să înăbușe revolta. Tudor Vladimirescu este în cele din urmă asasinat.</t>
+          <t>Unul dintre cele mai distructive conflicte ale secolului pentru spațiul românesc: Moldova și Țara Românească sunt complet ocupate de armatele țariste, iar bătăliile importante de la Larga și Cahul se dau pe teritoriul basarabean de atunci. Pacea de la Kuciuk-Kainargi (1774) retrocedează formal Principatele otomanilor, dar Rusia obține dreptul de a interveni în protejarea creștinilor; în 1775 Austria anexează nordul Moldovei (Bucovina).</t>
         </is>
       </c>
       <c r="R164" s="2" t="inlineStr">
         <is>
-          <t>Înăbușirea revoltei; sfârșitul lui Tudor Vladimirescu</t>
+          <t>Ocupație și distrugeri; dreptul rusesc de intervenție; anexarea Bucovinei</t>
         </is>
       </c>
       <c r="S164" s="2" t="inlineStr">
@@ -16045,12 +16045,12 @@
       </c>
       <c r="T164" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Bătăliile de la Larga și Cahul au avut loc în afara granițelor actuale ale României.</t>
         </is>
       </c>
       <c r="U164" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XIX d.Hr.</t>
+          <t>batalii.csv — sec. XVIII d.Hr., pct. 4</t>
         </is>
       </c>
     </row>
@@ -16062,41 +16062,41 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Războiul Ruso-Turc (1828–1829) și ocuparea Principatelor</t>
+          <t>Războiul Ruso-Austro-Turc (1787–1792) și bătăliile de la Focșani și Râmnicu Sărat</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Război / ocupație</t>
+          <t>Război / bătălii</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>1828</t>
+          <t>1787</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>1829</t>
+          <t>1792</t>
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>1828</v>
+        <v>1787</v>
       </c>
       <c r="G165" s="2" t="n">
-        <v>1829</v>
+        <v>1792</v>
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>sec. XIX d.Hr.</t>
+          <t>sec. XVIII d.Hr.</t>
         </is>
       </c>
       <c r="I165" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J165" s="2" t="inlineStr">
         <is>
-          <t>Principatele Române (Moldova și Țara Românească)</t>
+          <t>București, Iași, Focșani, Râmnicu Sărat</t>
         </is>
       </c>
       <c r="K165" s="2" t="n">
@@ -16104,48 +16104,48 @@
       </c>
       <c r="L165" s="2" t="inlineStr">
         <is>
+          <t>Ilfov / Iași / Vrancea / Buzău</t>
+        </is>
+      </c>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>Țara Românească / Moldova</t>
+        </is>
+      </c>
+      <c r="N165" s="2" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="O165" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="P165" s="2" t="inlineStr">
+        <is>
+          <t>Rusia și Imperiul Habsburgic vs. Imperiul Otoman</t>
+        </is>
+      </c>
+      <c r="Q165" s="2" t="inlineStr">
+        <is>
+          <t>Alianța austro-rusă atacă Imperiul Otoman pe pământ românesc: Bucureștiul și Iașiul sunt ocupate militar de trupele aliate, iar generalul rus Suvorov obține victorii răsunătoare la Focșani (1789) și Râmnicu Sărat (1789). Războiul se încheie prin Pacea de la Șiștov (1791) cu Austria și Pacea de la Iași (1792) cu Rusia, când granița rusă ajunge pentru prima dată pe Nistru.</t>
+        </is>
+      </c>
+      <c r="R165" s="2" t="inlineStr">
+        <is>
+          <t>Ocupație militară; granița rusă pe Nistru; restabilirea suzeranității otomane</t>
+        </is>
+      </c>
+      <c r="S165" s="2" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
+      <c r="T165" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M165" s="2" t="inlineStr">
-        <is>
-          <t>Moldova / Țara Românească</t>
-        </is>
-      </c>
-      <c r="N165" s="2" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="O165" s="2" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="P165" s="2" t="inlineStr">
-        <is>
-          <t>Imperiul Rus vs. Imperiul Otoman</t>
-        </is>
-      </c>
-      <c r="Q165" s="2" t="inlineStr">
-        <is>
-          <t>Principatele sunt ocupate de armata țaristă. Tratatul de la Adrianopol aduce modificări economice și politice majore (instituirea Regulamentelor Organice) și retrocedează Țării Românești cetățile dunărene: Brăila, Giurgiu și Turnu.</t>
-        </is>
-      </c>
-      <c r="R165" s="2" t="inlineStr">
-        <is>
-          <t>Ocupație rusească; Regulamentele Organice; recâștigarea cetăților dunărene</t>
-        </is>
-      </c>
-      <c r="S165" s="2" t="inlineStr">
-        <is>
-          <t>Da</t>
-        </is>
-      </c>
-      <c r="T165" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="U165" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XIX d.Hr.</t>
+          <t>batalii.csv — sec. XVIII d.Hr., pct. 5</t>
         </is>
       </c>
     </row>
@@ -16157,29 +16157,29 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Revoluția de la 1848–1849 din Transilvania (război civil)</t>
+          <t>Războiul Ruso-Turc (1806–1812) și anexarea Basarabiei</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Revoluție / război civil</t>
+          <t>Război</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>1848</t>
+          <t>1806</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>1849</t>
+          <t>1812</t>
         </is>
       </c>
       <c r="F166" s="2" t="n">
-        <v>1848</v>
+        <v>1806</v>
       </c>
       <c r="G166" s="2" t="n">
-        <v>1849</v>
+        <v>1812</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -16191,7 +16191,7 @@
       </c>
       <c r="J166" s="2" t="inlineStr">
         <is>
-          <t>Transilvania: Munții Apuseni și diverse localități transilvănene</t>
+          <t>Moldova (dintre Prut și Nistru) și Țara Românească</t>
         </is>
       </c>
       <c r="K166" s="2" t="n">
@@ -16204,28 +16204,28 @@
       </c>
       <c r="M166" s="2" t="inlineStr">
         <is>
-          <t>Transilvania</t>
+          <t>Moldova</t>
         </is>
       </c>
       <c r="N166" s="2" t="n">
-        <v>46.3</v>
+        <v>47</v>
       </c>
       <c r="O166" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="P166" s="2" t="inlineStr">
         <is>
-          <t>Revoluționarii maghiari vs. românii transilvăneni (Avram Iancu, aliați temporar cu Casa de Habsburg)</t>
+          <t>Imperiul Rus vs. Imperiul Otoman (principatele române ca teatru de război)</t>
         </is>
       </c>
       <c r="Q166" s="2" t="inlineStr">
         <is>
-          <t>Revoluția degenerază într-un război civil sângeros între revoluționarii maghiari (care doreau unirea Transilvaniei cu Ungaria) și românii transilvăneni conduși de Avram Iancu, care apărau drepturile naționale ale românilor. Confruntările armate au loc în Munții Apuseni și în diverse localități, până la intervenția trupelor țariste, care înfrâng armata maghiară.</t>
+          <t>Spațiul românesc este teatru de operațiuni sau ocupat militar: războiul se încheie cu Pacea de la București, prin care Imperiul Rus anexează jumătatea de est a Moldovei — teritoriul dintre Prut și Nistru, numit ulterior Basarabia.</t>
         </is>
       </c>
       <c r="R166" s="2" t="inlineStr">
         <is>
-          <t>Înfrângerea armatei maghiare de către intervenția țaristă; urmări pentru națiunea română</t>
+          <t>Anexarea Basarabiei de către Imperiul Rus</t>
         </is>
       </c>
       <c r="S166" s="2" t="inlineStr">
@@ -16235,7 +16235,7 @@
       </c>
       <c r="T166" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Moștenirea teritorială a evenimentului privește și Republica Moldova de azi.</t>
         </is>
       </c>
       <c r="U166" s="2" t="inlineStr">
@@ -16252,29 +16252,29 @@
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Lupta de la Brad (1849)</t>
+          <t>Revoluția lui Tudor Vladimirescu (1821)</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>Bătălie</t>
+          <t>Revoltă / război intern</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>1849-02</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>1849-02</t>
+          <t>1821</t>
         </is>
       </c>
       <c r="F167" s="2" t="n">
-        <v>1849</v>
+        <v>1821</v>
       </c>
       <c r="G167" s="2" t="n">
-        <v>1849</v>
+        <v>1821</v>
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
@@ -16286,41 +16286,41 @@
       </c>
       <c r="J167" s="2" t="inlineStr">
         <is>
-          <t>Brad (județul Hunedoara), Munții Apuseni</t>
+          <t>Țara Românească: Gorj, Oltenia, București</t>
         </is>
       </c>
       <c r="K167" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L167" s="2" t="inlineStr">
         <is>
-          <t>Hunedoara</t>
+          <t>Gorj / Dolj / Ilfov</t>
         </is>
       </c>
       <c r="M167" s="2" t="inlineStr">
         <is>
-          <t>Transilvania</t>
+          <t>Țara Românească</t>
         </is>
       </c>
       <c r="N167" s="2" t="n">
-        <v>46.12</v>
+        <v>44.8</v>
       </c>
       <c r="O167" s="2" t="n">
-        <v>22.18</v>
+        <v>23.5</v>
       </c>
       <c r="P167" s="2" t="inlineStr">
         <is>
-          <t>Românii din Munții Apuseni (Avram Iancu) vs. revoluționarii maghiari</t>
+          <t>Pandurii lui Tudor Vladimirescu și eteriștii (Alexandru Ipsilanti) vs. Imperiul Otoman</t>
         </is>
       </c>
       <c r="Q167" s="2" t="inlineStr">
         <is>
-          <t>În confruntările din Munții Apuseni, moții conduși de Avram Iancu obțin o victorie importantă la Brad, consolidând controlul românesc asupra zonei și respingând ofensiva revoluționarilor maghiari.</t>
+          <t>Mișcare socială și națională puternică în Țara Românească: se dau lupte între pandurii lui Tudor Vladimirescu, eteriștii (revoluționarii greci conduși de Alexandru Ipsilanti, care acționau tot pe teritoriu românesc) și armatele otomane venite să înăbușe revolta. Tudor Vladimirescu este în cele din urmă asasinat.</t>
         </is>
       </c>
       <c r="R167" s="2" t="inlineStr">
         <is>
-          <t>Victorie a moților la Brad</t>
+          <t>Înăbușirea revoltei; sfârșitul lui Tudor Vladimirescu</t>
         </is>
       </c>
       <c r="S167" s="2" t="inlineStr">
@@ -16330,12 +16330,12 @@
       </c>
       <c r="T167" s="2" t="inlineStr">
         <is>
-          <t>Se desfășoară în contextul războiului civil din Transilvania (1848–1849).</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U167" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XIX d.Hr. (completare)</t>
+          <t>batalii.csv — sec. XIX d.Hr.</t>
         </is>
       </c>
     </row>
@@ -16347,29 +16347,29 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Luptele de la Abrud (1849)</t>
+          <t>Războiul Ruso-Turc (1828–1829) și ocuparea Principatelor</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Bătălie</t>
+          <t>Război / ocupație</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>1849-05</t>
+          <t>1828</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>1849-05</t>
+          <t>1829</t>
         </is>
       </c>
       <c r="F168" s="2" t="n">
-        <v>1849</v>
+        <v>1828</v>
       </c>
       <c r="G168" s="2" t="n">
-        <v>1849</v>
+        <v>1829</v>
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
@@ -16381,41 +16381,41 @@
       </c>
       <c r="J168" s="2" t="inlineStr">
         <is>
-          <t>Abrud (județul Alba), Munții Apuseni</t>
+          <t>Principatele Române (Moldova și Țara Românească)</t>
         </is>
       </c>
       <c r="K168" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L168" s="2" t="inlineStr">
         <is>
-          <t>Alba</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M168" s="2" t="inlineStr">
         <is>
-          <t>Transilvania</t>
+          <t>Moldova / Țara Românească</t>
         </is>
       </c>
       <c r="N168" s="2" t="n">
-        <v>46.28</v>
+        <v>46.5</v>
       </c>
       <c r="O168" s="2" t="n">
-        <v>23.09</v>
+        <v>26.5</v>
       </c>
       <c r="P168" s="2" t="inlineStr">
         <is>
-          <t>Românii din Munții Apuseni (Avram Iancu) vs. revoluționarii maghiari (Ioan Hora, generalul Kemeny)</t>
+          <t>Imperiul Rus vs. Imperiul Otoman</t>
         </is>
       </c>
       <c r="Q168" s="2" t="inlineStr">
         <is>
-          <t>În cadrul războiului civil din Transilvania, Avram Iancu apără cu moții săi localitatea Abrud repetat, provocând înfrângeri grele armatei revoluționare maghiare, care încerca să ocupe Munții Apuseni. Luptele de la Abrud sunt printre cele mai celebre confruntări ale Revoluției de la 1848–1849 din Ardeal.</t>
+          <t>Principatele sunt ocupate de armata țaristă. Tratatul de la Adrianopol aduce modificări economice și politice majore (instituirea Regulamentelor Organice) și retrocedează Țării Românești cetățile dunărene: Brăila, Giurgiu și Turnu.</t>
         </is>
       </c>
       <c r="R168" s="2" t="inlineStr">
         <is>
-          <t>Victorie a moților lui Avram Iancu; apărarea Munților Apuseni</t>
+          <t>Ocupație rusească; Regulamentele Organice; recâștigarea cetăților dunărene</t>
         </is>
       </c>
       <c r="S168" s="2" t="inlineStr">
@@ -16425,12 +16425,12 @@
       </c>
       <c r="T168" s="2" t="inlineStr">
         <is>
-          <t>Se desfășoară în contextul războiului civil din Transilvania (1848–1849).</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U168" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XIX d.Hr. (completare)</t>
+          <t>batalii.csv — sec. XIX d.Hr.</t>
         </is>
       </c>
     </row>
@@ -16442,29 +16442,29 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Războiul Crimeii — ocuparea Principatelor (1853–1856)</t>
+          <t>Revoluția de la 1848–1849 din Transilvania (război civil)</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>Război / ocupații</t>
+          <t>Revoluție / război civil</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>1853</t>
+          <t>1848</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>1856</t>
+          <t>1849</t>
         </is>
       </c>
       <c r="F169" s="2" t="n">
-        <v>1853</v>
+        <v>1848</v>
       </c>
       <c r="G169" s="2" t="n">
-        <v>1856</v>
+        <v>1849</v>
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
@@ -16476,7 +16476,7 @@
       </c>
       <c r="J169" s="2" t="inlineStr">
         <is>
-          <t>Principatele Române (Moldova și Țara Românească)</t>
+          <t>Transilvania: Munții Apuseni și diverse localități transilvănene</t>
         </is>
       </c>
       <c r="K169" s="2" t="n">
@@ -16489,28 +16489,28 @@
       </c>
       <c r="M169" s="2" t="inlineStr">
         <is>
-          <t>Moldova / Țara Românească</t>
+          <t>Transilvania</t>
         </is>
       </c>
       <c r="N169" s="2" t="n">
-        <v>46.5</v>
+        <v>46.3</v>
       </c>
       <c r="O169" s="2" t="n">
-        <v>26.5</v>
+        <v>23</v>
       </c>
       <c r="P169" s="2" t="inlineStr">
         <is>
-          <t>Imperiul Rus vs. Imperiul Otoman (cu ocupări austriece și otomane de siguranță)</t>
+          <t>Revoluționarii maghiari vs. românii transilvăneni (Avram Iancu, aliați temporar cu Casa de Habsburg)</t>
         </is>
       </c>
       <c r="Q169" s="2" t="inlineStr">
         <is>
-          <t>Conflictul începe prin ocuparea Principatelor Române de către trupele rusești, urmată apoi de o ocupație austriacă și otomană de siguranță. Deși luptele mari se mută în Crimeea, teritoriul românesc este direct afectat de ocupații și rechiziții.</t>
+          <t>Revoluția degenerază într-un război civil sângeros între revoluționarii maghiari (care doreau unirea Transilvaniei cu Ungaria) și românii transilvăneni conduși de Avram Iancu, care apărau drepturile naționale ale românilor. Confruntările armate au loc în Munții Apuseni și în diverse localități, până la intervenția trupelor țariste, care înfrâng armata maghiară.</t>
         </is>
       </c>
       <c r="R169" s="2" t="inlineStr">
         <is>
-          <t>Ocupații succesive; restrângerea influenței ruse în principate</t>
+          <t>Înfrângerea armatei maghiare de către intervenția țaristă; urmări pentru națiunea română</t>
         </is>
       </c>
       <c r="S169" s="2" t="inlineStr">
@@ -16537,7 +16537,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Plevna</t>
+          <t>Lupta de la Brad (1849)</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
@@ -16547,19 +16547,19 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>1877-07</t>
+          <t>1849-02</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>1877-12-10</t>
+          <t>1849-02</t>
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>1877</v>
+        <v>1849</v>
       </c>
       <c r="G170" s="2" t="n">
-        <v>1877</v>
+        <v>1849</v>
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
@@ -16571,51 +16571,51 @@
       </c>
       <c r="J170" s="2" t="inlineStr">
         <is>
-          <t>Plevna (azi Pleven, Bulgaria)</t>
+          <t>Brad (județul Hunedoara), Munții Apuseni</t>
         </is>
       </c>
       <c r="K170" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L170" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Hunedoara</t>
         </is>
       </c>
       <c r="M170" s="2" t="inlineStr">
         <is>
-          <t>Bulgaria (în afara actualelor granițe)</t>
+          <t>Transilvania</t>
         </is>
       </c>
       <c r="N170" s="2" t="n">
-        <v>43.42</v>
+        <v>46.12</v>
       </c>
       <c r="O170" s="2" t="n">
-        <v>24.62</v>
+        <v>22.18</v>
       </c>
       <c r="P170" s="2" t="inlineStr">
         <is>
-          <t>România și Imperiul Țarist vs. Imperiul Otoman (Osman Pașa)</t>
+          <t>Românii din Munții Apuseni (Avram Iancu) vs. revoluționarii maghiari</t>
         </is>
       </c>
       <c r="Q170" s="2" t="inlineStr">
         <is>
-          <t>Asediul de la Plevna este cea mai sângeroasă confruntare a Războiului de Independență: trupele române și ruse asediază și înfrâng garnizoana otomană a lui Osman Pașa, care capitulează la 10 decembrie 1877. Victoria contribuie decisiv la obținerea independenței României.</t>
+          <t>În confruntările din Munții Apuseni, moții conduși de Avram Iancu obțin o victorie importantă la Brad, consolidând controlul românesc asupra zonei și respingând ofensiva revoluționarilor maghiari.</t>
         </is>
       </c>
       <c r="R170" s="2" t="inlineStr">
         <is>
-          <t>Victoria ruso-română; capitularea garnizoanei otomane</t>
+          <t>Victorie a moților la Brad</t>
         </is>
       </c>
       <c r="S170" s="2" t="inlineStr">
         <is>
-          <t>Nu (context regional)</t>
+          <t>Da</t>
         </is>
       </c>
       <c r="T170" s="2" t="inlineStr">
         <is>
-          <t>Bătălia s-a desfășurat în afara teritoriului actual al României, dar este legată direct de Războiul de Independență.</t>
+          <t>Se desfășoară în contextul războiului civil din Transilvania (1848–1849).</t>
         </is>
       </c>
       <c r="U170" s="2" t="inlineStr">
@@ -16632,7 +16632,7 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Luptele de la Grivița (1877)</t>
+          <t>Luptele de la Abrud (1849)</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
@@ -16642,19 +16642,19 @@
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>1877-08-30</t>
+          <t>1849-05</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>1877-08-30</t>
+          <t>1849-05</t>
         </is>
       </c>
       <c r="F171" s="2" t="n">
-        <v>1877</v>
+        <v>1849</v>
       </c>
       <c r="G171" s="2" t="n">
-        <v>1877</v>
+        <v>1849</v>
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
@@ -16666,51 +16666,51 @@
       </c>
       <c r="J171" s="2" t="inlineStr">
         <is>
-          <t>Reduta Grivița, lângă Plevna (azi Pleven, Bulgaria)</t>
+          <t>Abrud (județul Alba), Munții Apuseni</t>
         </is>
       </c>
       <c r="K171" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L171" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Alba</t>
         </is>
       </c>
       <c r="M171" s="2" t="inlineStr">
         <is>
-          <t>Bulgaria (în afara actualelor granițe)</t>
+          <t>Transilvania</t>
         </is>
       </c>
       <c r="N171" s="2" t="n">
-        <v>43.4</v>
+        <v>46.28</v>
       </c>
       <c r="O171" s="2" t="n">
-        <v>24.6</v>
+        <v>23.09</v>
       </c>
       <c r="P171" s="2" t="inlineStr">
         <is>
-          <t>România (armata română) vs. Imperiul Otoman</t>
+          <t>Românii din Munții Apuseni (Avram Iancu) vs. revoluționarii maghiari (Ioan Hora, generalul Kemeny)</t>
         </is>
       </c>
       <c r="Q171" s="2" t="inlineStr">
         <is>
-          <t>Atacul românilor asupra redutei Grivița de la Plevna este una dintre cele mai eroice fapte de arme ale Războiului de Independență, soldată cu cucerirea redutei după lupte extrem de sângeroase, celebrată în cultura românească.</t>
+          <t>În cadrul războiului civil din Transilvania, Avram Iancu apără cu moții săi localitatea Abrud repetat, provocând înfrângeri grele armatei revoluționare maghiare, care încerca să ocupe Munții Apuseni. Luptele de la Abrud sunt printre cele mai celebre confruntări ale Revoluției de la 1848–1849 din Ardeal.</t>
         </is>
       </c>
       <c r="R171" s="2" t="inlineStr">
         <is>
-          <t>Cucerirea redutei Grivița de către armata română</t>
+          <t>Victorie a moților lui Avram Iancu; apărarea Munților Apuseni</t>
         </is>
       </c>
       <c r="S171" s="2" t="inlineStr">
         <is>
-          <t>Nu (context regional)</t>
+          <t>Da</t>
         </is>
       </c>
       <c r="T171" s="2" t="inlineStr">
         <is>
-          <t>În afara granițelor actuale; parte din Războiul de Independență.</t>
+          <t>Se desfășoară în contextul războiului civil din Transilvania (1848–1849).</t>
         </is>
       </c>
       <c r="U171" s="2" t="inlineStr">
@@ -16727,29 +16727,29 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Războiul de Independență (Russo-Turc 1877–1878)</t>
+          <t>Războiul Crimeii — ocuparea Principatelor (1853–1856)</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Război</t>
+          <t>Război / ocupații</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>1877-04</t>
+          <t>1853</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>1878</t>
+          <t>1856</t>
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>1877</v>
+        <v>1853</v>
       </c>
       <c r="G172" s="2" t="n">
-        <v>1878</v>
+        <v>1856</v>
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
@@ -16761,7 +16761,7 @@
       </c>
       <c r="J172" s="2" t="inlineStr">
         <is>
-          <t>Trecerea Dunării (Zimnicea) și luptele din Bulgaria (Plevna, Grivița, Rahova, Vidin)</t>
+          <t>Principatele Române (Moldova și Țara Românească)</t>
         </is>
       </c>
       <c r="K172" s="2" t="n">
@@ -16769,43 +16769,43 @@
       </c>
       <c r="L172" s="2" t="inlineStr">
         <is>
-          <t>Teleorman</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M172" s="2" t="inlineStr">
         <is>
-          <t>Țara Românească / Balcani</t>
+          <t>Moldova / Țara Românească</t>
         </is>
       </c>
       <c r="N172" s="2" t="n">
-        <v>43.65</v>
+        <v>46.5</v>
       </c>
       <c r="O172" s="2" t="n">
-        <v>25.37</v>
+        <v>26.5</v>
       </c>
       <c r="P172" s="2" t="inlineStr">
         <is>
-          <t>România (domnitorul Carol I) și Imperiul Rus vs. Imperiul Otoman</t>
+          <t>Imperiul Rus vs. Imperiul Otoman (cu ocupări austriece și otomane de siguranță)</t>
         </is>
       </c>
       <c r="Q172" s="2" t="inlineStr">
         <is>
-          <t>Armata rusă traversează România pentru a ataca Imperiul Otoman; România se alătură militar Rusiei, iar trupele conduse de Carol I au un rol decisiv în asediile de la Plevna, Grivița, Rahova și Vidin. Conflictul consfințește independența de stat a României.</t>
+          <t>Conflictul începe prin ocuparea Principatelor Române de către trupele rusești, urmată apoi de o ocupație austriacă și otomană de siguranță. Deși luptele mari se mută în Crimeea, teritoriul românesc este direct afectat de ocupații și rechiziții.</t>
         </is>
       </c>
       <c r="R172" s="2" t="inlineStr">
         <is>
-          <t>Independența României (1877–1878); recunoaștere internațională</t>
+          <t>Ocupații succesive; restrângerea influenței ruse în principate</t>
         </is>
       </c>
       <c r="S172" s="2" t="inlineStr">
         <is>
-          <t>Parțial (graniță/zona învecinată)</t>
+          <t>Da</t>
         </is>
       </c>
       <c r="T172" s="2" t="inlineStr">
         <is>
-          <t>Luptele principale au avut loc în afara granițelor actuale (Bulgaria); trecerea Dunării și mobilizarea s-au desfășurat pe teritoriul românesc.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U172" s="2" t="inlineStr">
@@ -16822,7 +16822,7 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Smârdan</t>
+          <t>Bătălia de la Plevna</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
@@ -16832,19 +16832,19 @@
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>1878-01-24</t>
+          <t>1877-07</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>1878-01-24</t>
+          <t>1877-12-10</t>
         </is>
       </c>
       <c r="F173" s="2" t="n">
-        <v>1878</v>
+        <v>1877</v>
       </c>
       <c r="G173" s="2" t="n">
-        <v>1878</v>
+        <v>1877</v>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
@@ -16856,7 +16856,7 @@
       </c>
       <c r="J173" s="2" t="inlineStr">
         <is>
-          <t>Smârdan, lângă Vidin (Bulgaria)</t>
+          <t>Plevna (azi Pleven, Bulgaria)</t>
         </is>
       </c>
       <c r="K173" s="2" t="n">
@@ -16873,24 +16873,24 @@
         </is>
       </c>
       <c r="N173" s="2" t="n">
-        <v>44</v>
+        <v>43.42</v>
       </c>
       <c r="O173" s="2" t="n">
-        <v>22.87</v>
+        <v>24.62</v>
       </c>
       <c r="P173" s="2" t="inlineStr">
         <is>
-          <t>România (armata română) vs. Imperiul Otoman</t>
+          <t>România și Imperiul Țarist vs. Imperiul Otoman (Osman Pașa)</t>
         </is>
       </c>
       <c r="Q173" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Smârdan, la 24 ianuarie 1878, este o victorie importantă a armatei române de la finalul Războiului de Independență, marcând ultima mare confruntare a campaniei de peste Dunăre și simbolizând închiderea campaniei victorioase.</t>
+          <t>Asediul de la Plevna este cea mai sângeroasă confruntare a Războiului de Independență: trupele române și ruse asediază și înfrâng garnizoana otomană a lui Osman Pașa, care capitulează la 10 decembrie 1877. Victoria contribuie decisiv la obținerea independenței României.</t>
         </is>
       </c>
       <c r="R173" s="2" t="inlineStr">
         <is>
-          <t>Victoria armatei române; finalul campaniei de peste Dunăre</t>
+          <t>Victoria ruso-română; capitularea garnizoanei otomane</t>
         </is>
       </c>
       <c r="S173" s="2" t="inlineStr">
@@ -16900,7 +16900,7 @@
       </c>
       <c r="T173" s="2" t="inlineStr">
         <is>
-          <t>În afara granițelor actuale; parte din Războiul de Independență.</t>
+          <t>Bătălia s-a desfășurat în afara teritoriului actual al României, dar este legată direct de Războiul de Independență.</t>
         </is>
       </c>
       <c r="U173" s="2" t="inlineStr">
@@ -16917,7 +16917,7 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Bazargic (1916)</t>
+          <t>Luptele de la Grivița (1877)</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
@@ -16927,31 +16927,31 @@
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>1916-09-05</t>
+          <t>1877-08-30</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>1916-09-07</t>
+          <t>1877-08-30</t>
         </is>
       </c>
       <c r="F174" s="2" t="n">
-        <v>1916</v>
+        <v>1877</v>
       </c>
       <c r="G174" s="2" t="n">
-        <v>1916</v>
+        <v>1877</v>
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>sec. XX d.Hr.</t>
+          <t>sec. XIX d.Hr.</t>
         </is>
       </c>
       <c r="I174" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J174" s="2" t="inlineStr">
         <is>
-          <t>Bazargic (azi Dobrici, Bulgaria) — Dobrogea de sud</t>
+          <t>Reduta Grivița, lângă Plevna (azi Pleven, Bulgaria)</t>
         </is>
       </c>
       <c r="K174" s="2" t="n">
@@ -16959,48 +16959,48 @@
       </c>
       <c r="L174" s="2" t="inlineStr">
         <is>
-          <t>Constanța</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M174" s="2" t="inlineStr">
         <is>
-          <t>Dobrogea</t>
+          <t>Bulgaria (în afara actualelor granițe)</t>
         </is>
       </c>
       <c r="N174" s="2" t="n">
-        <v>43.57</v>
+        <v>43.4</v>
       </c>
       <c r="O174" s="2" t="n">
-        <v>27.83</v>
+        <v>24.6</v>
       </c>
       <c r="P174" s="2" t="inlineStr">
         <is>
-          <t>România și Imperiul Țarist vs. Bulgaria și Imperiul German</t>
+          <t>România (armata română) vs. Imperiul Otoman</t>
         </is>
       </c>
       <c r="Q174" s="2" t="inlineStr">
         <is>
-          <t>În fața ofensivei bulgaro-germane în Dobrogea, trupele române și ruse sunt înfrânte la Bazargic (Dobrici), în prima mare bătălie de pe frontul dobrogean din campania din 1916. Înfrângerea contribuie la pierderea Dobrogei.</t>
+          <t>Atacul românilor asupra redutei Grivița de la Plevna este una dintre cele mai eroice fapte de arme ale Războiului de Independență, soldată cu cucerirea redutei după lupte extrem de sângeroase, celebrată în cultura românească.</t>
         </is>
       </c>
       <c r="R174" s="2" t="inlineStr">
         <is>
-          <t>Victoria forțelor bulgaro-germane; înaintarea în Dobrogea</t>
+          <t>Cucerirea redutei Grivița de către armata română</t>
         </is>
       </c>
       <c r="S174" s="2" t="inlineStr">
         <is>
-          <t>Parțial (graniță/zona învecinată)</t>
+          <t>Nu (context regional)</t>
         </is>
       </c>
       <c r="T174" s="2" t="inlineStr">
         <is>
-          <t>Bazargic se află la granița actuală dintre România și Bulgaria (Dobrogea de sud).</t>
+          <t>În afara granițelor actuale; parte din Războiul de Independență.</t>
         </is>
       </c>
       <c r="U174" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
+          <t>batalii.csv — sec. XIX d.Hr. (completare)</t>
         </is>
       </c>
     </row>
@@ -17012,41 +17012,41 @@
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Brașov (1916)</t>
+          <t>Războiul de Independență (Russo-Turc 1877–1878)</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>Bătălie</t>
+          <t>Război</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>1916-10-07</t>
+          <t>1877-04</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>1916-10-08</t>
+          <t>1878</t>
         </is>
       </c>
       <c r="F175" s="2" t="n">
-        <v>1916</v>
+        <v>1877</v>
       </c>
       <c r="G175" s="2" t="n">
-        <v>1916</v>
+        <v>1878</v>
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>sec. XX d.Hr.</t>
+          <t>sec. XIX d.Hr.</t>
         </is>
       </c>
       <c r="I175" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J175" s="2" t="inlineStr">
         <is>
-          <t>Brașov și Țara Bârsei (județul Brașov)</t>
+          <t>Trecerea Dunării (Zimnicea) și luptele din Bulgaria (Plevna, Grivița, Rahova, Vidin)</t>
         </is>
       </c>
       <c r="K175" s="2" t="n">
@@ -17054,48 +17054,48 @@
       </c>
       <c r="L175" s="2" t="inlineStr">
         <is>
-          <t>Brașov</t>
+          <t>Teleorman</t>
         </is>
       </c>
       <c r="M175" s="2" t="inlineStr">
         <is>
-          <t>Transilvania</t>
+          <t>Țara Românească / Balcani</t>
         </is>
       </c>
       <c r="N175" s="2" t="n">
-        <v>45.66</v>
+        <v>43.65</v>
       </c>
       <c r="O175" s="2" t="n">
-        <v>25.61</v>
+        <v>25.37</v>
       </c>
       <c r="P175" s="2" t="inlineStr">
         <is>
-          <t>România (Armata a 2-a) vs. Imperiul German (Armata a 9-a)</t>
+          <t>România (domnitorul Carol I) și Imperiul Rus vs. Imperiul Otoman</t>
         </is>
       </c>
       <c r="Q175" s="2" t="inlineStr">
         <is>
-          <t>Armata română a 2-a încercă să oprească înaintarea Armatei a 9-a germane prin Țara Bârsei, dar este înfrântă și se retrage din Brașov, ultima mare confruntare din ofensiva germană din Transilvania de la sfârșitul anului 1916.</t>
+          <t>Armata rusă traversează România pentru a ataca Imperiul Otoman; România se alătură militar Rusiei, iar trupele conduse de Carol I au un rol decisiv în asediile de la Plevna, Grivița, Rahova și Vidin. Conflictul consfințește independența de stat a României.</t>
         </is>
       </c>
       <c r="R175" s="2" t="inlineStr">
         <is>
-          <t>Victorie a Puterilor Centrale; retragerea Armatei a 2-a</t>
+          <t>Independența României (1877–1878); recunoaștere internațională</t>
         </is>
       </c>
       <c r="S175" s="2" t="inlineStr">
         <is>
-          <t>Da</t>
+          <t>Parțial (graniță/zona învecinată)</t>
         </is>
       </c>
       <c r="T175" s="2" t="inlineStr">
         <is>
-          <t>Parte din operația de apărare a trecătorilor din 1916.</t>
+          <t>Luptele principale au avut loc în afara granițelor actuale (Bulgaria); trecerea Dunării și mobilizarea s-au desfășurat pe teritoriul românesc.</t>
         </is>
       </c>
       <c r="U175" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
+          <t>batalii.csv — sec. XIX d.Hr.</t>
         </is>
       </c>
     </row>
@@ -17107,7 +17107,7 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Predeal (1916)</t>
+          <t>Bătălia de la Smârdan</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
@@ -17117,80 +17117,80 @@
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>1916-10</t>
+          <t>1878-01-24</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>1916-10</t>
+          <t>1878-01-24</t>
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>1916</v>
+        <v>1878</v>
       </c>
       <c r="G176" s="2" t="n">
-        <v>1916</v>
+        <v>1878</v>
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>sec. XX d.Hr.</t>
+          <t>sec. XIX d.Hr.</t>
         </is>
       </c>
       <c r="I176" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J176" s="2" t="inlineStr">
         <is>
-          <t>Predeal, trecătoarea din Carpații Meridionali (județul Brașov)</t>
+          <t>Smârdan, lângă Vidin (Bulgaria)</t>
         </is>
       </c>
       <c r="K176" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L176" s="2" t="inlineStr">
         <is>
-          <t>Brașov</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M176" s="2" t="inlineStr">
         <is>
-          <t>Transilvania / Muntenia</t>
+          <t>Bulgaria (în afara actualelor granițe)</t>
         </is>
       </c>
       <c r="N176" s="2" t="n">
-        <v>45.5</v>
+        <v>44</v>
       </c>
       <c r="O176" s="2" t="n">
-        <v>25.58</v>
+        <v>22.87</v>
       </c>
       <c r="P176" s="2" t="inlineStr">
         <is>
-          <t>România vs. Imperiul German și Austro-Ungaria</t>
+          <t>România (armata română) vs. Imperiul Otoman</t>
         </is>
       </c>
       <c r="Q176" s="2" t="inlineStr">
         <is>
-          <t>În confruntările pentru trecătoarea Predeal, trupele române rezistă eroic, dar sunt nevoite să se retragă spre zona Bran–Câmpulung, în cadrul operației de apărare a trecătorilor din Carpați în campania din 1916.</t>
+          <t>Bătălia de la Smârdan, la 24 ianuarie 1878, este o victorie importantă a armatei române de la finalul Războiului de Independență, marcând ultima mare confruntare a campaniei de peste Dunăre și simbolizând închiderea campaniei victorioase.</t>
         </is>
       </c>
       <c r="R176" s="2" t="inlineStr">
         <is>
-          <t>Depășirea trecătorii de către Puterile Centrale</t>
+          <t>Victoria armatei române; finalul campaniei de peste Dunăre</t>
         </is>
       </c>
       <c r="S176" s="2" t="inlineStr">
         <is>
-          <t>Da</t>
+          <t>Nu (context regional)</t>
         </is>
       </c>
       <c r="T176" s="2" t="inlineStr">
         <is>
-          <t>Parte din operația de apărare a trecătorilor din 1916.</t>
+          <t>În afara granițelor actuale; parte din Războiul de Independență.</t>
         </is>
       </c>
       <c r="U176" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
+          <t>batalii.csv — sec. XIX d.Hr. (completare)</t>
         </is>
       </c>
     </row>
@@ -17202,7 +17202,7 @@
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Sibiu (1916)</t>
+          <t>Bătălia de la Bazargic (1916)</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
@@ -17212,12 +17212,12 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>1916-09-26</t>
+          <t>1916-09-05</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>1916-09-29</t>
+          <t>1916-09-07</t>
         </is>
       </c>
       <c r="F177" s="2" t="n">
@@ -17236,7 +17236,7 @@
       </c>
       <c r="J177" s="2" t="inlineStr">
         <is>
-          <t>Sibiu și zona trecătorilor din Carpații Meridionali (județul Sibiu)</t>
+          <t>Bazargic (azi Dobrici, Bulgaria) — Dobrogea de sud</t>
         </is>
       </c>
       <c r="K177" s="2" t="n">
@@ -17244,43 +17244,43 @@
       </c>
       <c r="L177" s="2" t="inlineStr">
         <is>
-          <t>Sibiu</t>
+          <t>Constanța</t>
         </is>
       </c>
       <c r="M177" s="2" t="inlineStr">
         <is>
-          <t>Transilvania</t>
+          <t>Dobrogea</t>
         </is>
       </c>
       <c r="N177" s="2" t="n">
-        <v>45.8</v>
+        <v>43.57</v>
       </c>
       <c r="O177" s="2" t="n">
-        <v>24.15</v>
+        <v>27.83</v>
       </c>
       <c r="P177" s="2" t="inlineStr">
         <is>
-          <t>România vs. Imperiul German și Austro-Ungaria</t>
+          <t>România și Imperiul Țarist vs. Bulgaria și Imperiul German</t>
         </is>
       </c>
       <c r="Q177" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Sibiu face parte din apărarea trecătorilor din Carpați: forțele Puterilor Centrale, venite din Transilvania, împing armata română și pătrund în zona Sibiu–Turnu Roșu, deschizând drumul spre sud.</t>
+          <t>În fața ofensivei bulgaro-germane în Dobrogea, trupele române și ruse sunt înfrânte la Bazargic (Dobrici), în prima mare bătălie de pe frontul dobrogean din campania din 1916. Înfrângerea contribuie la pierderea Dobrogei.</t>
         </is>
       </c>
       <c r="R177" s="2" t="inlineStr">
         <is>
-          <t>Victorie a Puterilor Centrale; depășirea apărării române</t>
+          <t>Victoria forțelor bulgaro-germane; înaintarea în Dobrogea</t>
         </is>
       </c>
       <c r="S177" s="2" t="inlineStr">
         <is>
-          <t>Da</t>
+          <t>Parțial (graniță/zona învecinată)</t>
         </is>
       </c>
       <c r="T177" s="2" t="inlineStr">
         <is>
-          <t>Parte din operația de apărare a trecătorilor din 1916.</t>
+          <t>Bazargic se află la granița actuală dintre România și Bulgaria (Dobrogea de sud).</t>
         </is>
       </c>
       <c r="U177" s="2" t="inlineStr">
@@ -17297,7 +17297,7 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Turtucaia</t>
+          <t>Bătălia de la Brașov (1916)</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
@@ -17307,12 +17307,12 @@
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>1916-09-02</t>
+          <t>1916-10-07</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>1916-09-06</t>
+          <t>1916-10-08</t>
         </is>
       </c>
       <c r="F178" s="2" t="n">
@@ -17331,7 +17331,7 @@
       </c>
       <c r="J178" s="2" t="inlineStr">
         <is>
-          <t>Turtucaia (azi Tutrakan, Bulgaria) — pe malul drept al Dunării, în fața Dobrogei</t>
+          <t>Brașov și Țara Bârsei (județul Brașov)</t>
         </is>
       </c>
       <c r="K178" s="2" t="n">
@@ -17339,48 +17339,48 @@
       </c>
       <c r="L178" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Brașov</t>
         </is>
       </c>
       <c r="M178" s="2" t="inlineStr">
         <is>
-          <t>Dobrogea (graniță)</t>
+          <t>Transilvania</t>
         </is>
       </c>
       <c r="N178" s="2" t="n">
-        <v>44.05</v>
+        <v>45.66</v>
       </c>
       <c r="O178" s="2" t="n">
-        <v>26.62</v>
+        <v>25.61</v>
       </c>
       <c r="P178" s="2" t="inlineStr">
         <is>
-          <t>România (garnizoana Turtucaia) vs. Bulgaria și Imperiul German</t>
+          <t>România (Armata a 2-a) vs. Imperiul German (Armata a 9-a)</t>
         </is>
       </c>
       <c r="Q178" s="2" t="inlineStr">
         <is>
-          <t>Înfrângere severă a trupelor române în fața armatei bulgaro-germane, care deschide drumul inamicului spre Dobrogea. Una dintre cele mai mari catastrofe militare ale românilor în Primul Război Mondial.</t>
+          <t>Armata română a 2-a încercă să oprească înaintarea Armatei a 9-a germane prin Țara Bârsei, dar este înfrântă și se retrage din Brașov, ultima mare confruntare din ofensiva germană din Transilvania de la sfârșitul anului 1916.</t>
         </is>
       </c>
       <c r="R178" s="2" t="inlineStr">
         <is>
-          <t>Înfrângere românească; ocuparea Dobrogei</t>
+          <t>Victorie a Puterilor Centrale; retragerea Armatei a 2-a</t>
         </is>
       </c>
       <c r="S178" s="2" t="inlineStr">
         <is>
-          <t>Nu (context regional)</t>
+          <t>Da</t>
         </is>
       </c>
       <c r="T178" s="2" t="inlineStr">
         <is>
-          <t>Turtucaia este azi în Bulgaria, imediat la frontiera cu România.</t>
+          <t>Parte din operația de apărare a trecătorilor din 1916.</t>
         </is>
       </c>
       <c r="U178" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr.</t>
+          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
         </is>
       </c>
     </row>
@@ -17392,7 +17392,7 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Târgu Jiu (1916)</t>
+          <t>Bătălia de la Predeal (1916)</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
@@ -17402,12 +17402,12 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>1916-11-16</t>
+          <t>1916-10</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>1916-11-17</t>
+          <t>1916-10</t>
         </is>
       </c>
       <c r="F179" s="2" t="n">
@@ -17426,7 +17426,7 @@
       </c>
       <c r="J179" s="2" t="inlineStr">
         <is>
-          <t>Târgu Jiu (județul Gorj)</t>
+          <t>Predeal, trecătoarea din Carpații Meridionali (județul Brașov)</t>
         </is>
       </c>
       <c r="K179" s="2" t="n">
@@ -17434,33 +17434,33 @@
       </c>
       <c r="L179" s="2" t="inlineStr">
         <is>
-          <t>Gorj</t>
+          <t>Brașov</t>
         </is>
       </c>
       <c r="M179" s="2" t="inlineStr">
         <is>
-          <t>Oltenia</t>
+          <t>Transilvania / Muntenia</t>
         </is>
       </c>
       <c r="N179" s="2" t="n">
-        <v>45.04</v>
+        <v>45.5</v>
       </c>
       <c r="O179" s="2" t="n">
-        <v>23.27</v>
+        <v>25.58</v>
       </c>
       <c r="P179" s="2" t="inlineStr">
         <is>
-          <t>România vs. Imperiul German (armata lui Falkenhayn)</t>
+          <t>România vs. Imperiul German și Austro-Ungaria</t>
         </is>
       </c>
       <c r="Q179" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Târgu Jiu are loc în cadrul apărării Olteniei: trupele române, după lupte grele pe Valea Jiului, încearcă să oprească înaintarea germană, dar orașul cade în mâinile Puterilor Centrale, pregătind marea bătălie de la Neajlov–Argeș și ocuparea Bucureștiului.</t>
+          <t>În confruntările pentru trecătoarea Predeal, trupele române rezistă eroic, dar sunt nevoite să se retragă spre zona Bran–Câmpulung, în cadrul operației de apărare a trecătorilor din Carpați în campania din 1916.</t>
         </is>
       </c>
       <c r="R179" s="2" t="inlineStr">
         <is>
-          <t>Victorie a Puterilor Centrale; căderea Târgu Jiului</t>
+          <t>Depășirea trecătorii de către Puterile Centrale</t>
         </is>
       </c>
       <c r="S179" s="2" t="inlineStr">
@@ -17470,7 +17470,7 @@
       </c>
       <c r="T179" s="2" t="inlineStr">
         <is>
-          <t>Parte din a doua bătălie de pe Valea Jiului și din apărarea Olteniei.</t>
+          <t>Parte din operația de apărare a trecătorilor din 1916.</t>
         </is>
       </c>
       <c r="U179" s="2" t="inlineStr">
@@ -17487,7 +17487,7 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de pe Neajlov–Argeș (1916)</t>
+          <t>Bătălia de la Sibiu (1916)</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
@@ -17497,12 +17497,12 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>1916-11</t>
+          <t>1916-09-26</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>1916-12</t>
+          <t>1916-09-29</t>
         </is>
       </c>
       <c r="F180" s="2" t="n">
@@ -17521,7 +17521,7 @@
       </c>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>Zona râurilor Neajlov și Argeș, la sud de București</t>
+          <t>Sibiu și zona trecătorilor din Carpații Meridionali (județul Sibiu)</t>
         </is>
       </c>
       <c r="K180" s="2" t="n">
@@ -17529,33 +17529,33 @@
       </c>
       <c r="L180" s="2" t="inlineStr">
         <is>
-          <t>Giurgiu / Ilfov</t>
+          <t>Sibiu</t>
         </is>
       </c>
       <c r="M180" s="2" t="inlineStr">
         <is>
-          <t>Muntenia</t>
+          <t>Transilvania</t>
         </is>
       </c>
       <c r="N180" s="2" t="n">
-        <v>44.35</v>
+        <v>45.8</v>
       </c>
       <c r="O180" s="2" t="n">
-        <v>25.75</v>
+        <v>24.15</v>
       </c>
       <c r="P180" s="2" t="inlineStr">
         <is>
-          <t>România vs. Imperiul German (von Mackensen)</t>
+          <t>România vs. Imperiul German și Austro-Ungaria</t>
         </is>
       </c>
       <c r="Q180" s="2" t="inlineStr">
         <is>
-          <t>Ultima încercare majoră de a opri înaintarea Puterilor Centrale spre București; după această confruntare, capitala este ocupată.</t>
+          <t>Bătălia de la Sibiu face parte din apărarea trecătorilor din Carpați: forțele Puterilor Centrale, venite din Transilvania, împing armata română și pătrund în zona Sibiu–Turnu Roșu, deschizând drumul spre sud.</t>
         </is>
       </c>
       <c r="R180" s="2" t="inlineStr">
         <is>
-          <t>Înfrângere românească; ocuparea Bucureștiului</t>
+          <t>Victorie a Puterilor Centrale; depășirea apărării române</t>
         </is>
       </c>
       <c r="S180" s="2" t="inlineStr">
@@ -17565,12 +17565,12 @@
       </c>
       <c r="T180" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Parte din operația de apărare a trecătorilor din 1916.</t>
         </is>
       </c>
       <c r="U180" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr.</t>
+          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
         </is>
       </c>
     </row>
@@ -17582,7 +17582,7 @@
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de pe Valea Jiului (1916)</t>
+          <t>Bătălia de la Turtucaia</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
@@ -17592,12 +17592,12 @@
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>1916-10</t>
+          <t>1916-09-02</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>1916-11</t>
+          <t>1916-09-06</t>
         </is>
       </c>
       <c r="F181" s="2" t="n">
@@ -17616,7 +17616,7 @@
       </c>
       <c r="J181" s="2" t="inlineStr">
         <is>
-          <t>Valea Jiului (județele Gorj/Hunedoara)</t>
+          <t>Turtucaia (azi Tutrakan, Bulgaria) — pe malul drept al Dunării, în fața Dobrogei</t>
         </is>
       </c>
       <c r="K181" s="2" t="n">
@@ -17624,43 +17624,43 @@
       </c>
       <c r="L181" s="2" t="inlineStr">
         <is>
-          <t>Gorj / Hunedoara</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M181" s="2" t="inlineStr">
         <is>
-          <t>Oltenia</t>
+          <t>Dobrogea (graniță)</t>
         </is>
       </c>
       <c r="N181" s="2" t="n">
-        <v>45.35</v>
+        <v>44.05</v>
       </c>
       <c r="O181" s="2" t="n">
-        <v>23.15</v>
+        <v>26.62</v>
       </c>
       <c r="P181" s="2" t="inlineStr">
         <is>
-          <t>România vs. Imperiul German (armata lui Falkenhayn)</t>
+          <t>România (garnizoana Turtucaia) vs. Bulgaria și Imperiul German</t>
         </is>
       </c>
       <c r="Q181" s="2" t="inlineStr">
         <is>
-          <t>Confruntare violentă prin care s-a încercat, fără succes, oprirea înaintării Puterilor Centrale, venite dinspre Transilvania prin Valea Jiului, spre București.</t>
+          <t>Înfrângere severă a trupelor române în fața armatei bulgaro-germane, care deschide drumul inamicului spre Dobrogea. Una dintre cele mai mari catastrofe militare ale românilor în Primul Război Mondial.</t>
         </is>
       </c>
       <c r="R181" s="2" t="inlineStr">
         <is>
-          <t>Succes german inițial; depășirea apărării române</t>
+          <t>Înfrângere românească; ocuparea Dobrogei</t>
         </is>
       </c>
       <c r="S181" s="2" t="inlineStr">
         <is>
-          <t>Da</t>
+          <t>Nu (context regional)</t>
         </is>
       </c>
       <c r="T181" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Turtucaia este azi în Bulgaria, imediat la frontiera cu România.</t>
         </is>
       </c>
       <c r="U181" s="2" t="inlineStr">
@@ -17677,7 +17677,7 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de pe Valea Prahovei (1916)</t>
+          <t>Bătălia de la Târgu Jiu (1916)</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
@@ -17687,12 +17687,12 @@
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>1916-10-09</t>
+          <t>1916-11-16</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>1916-10-25</t>
+          <t>1916-11-17</t>
         </is>
       </c>
       <c r="F182" s="2" t="n">
@@ -17711,41 +17711,41 @@
       </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
-          <t>Valea Prahovei, în Carpații Meridionali (județul Prahova)</t>
+          <t>Târgu Jiu (județul Gorj)</t>
         </is>
       </c>
       <c r="K182" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L182" s="2" t="inlineStr">
         <is>
-          <t>Prahova</t>
+          <t>Gorj</t>
         </is>
       </c>
       <c r="M182" s="2" t="inlineStr">
         <is>
-          <t>Muntenia</t>
+          <t>Oltenia</t>
         </is>
       </c>
       <c r="N182" s="2" t="n">
-        <v>45.2</v>
+        <v>45.04</v>
       </c>
       <c r="O182" s="2" t="n">
-        <v>25.7</v>
+        <v>23.27</v>
       </c>
       <c r="P182" s="2" t="inlineStr">
         <is>
-          <t>România vs. Imperiul German și Austro-Ungaria</t>
+          <t>România vs. Imperiul German (armata lui Falkenhayn)</t>
         </is>
       </c>
       <c r="Q182" s="2" t="inlineStr">
         <is>
-          <t>Confruntări violente pe valea Prahovei, una dintre principalele căi de acces spre București: armata română încearcă să blocheze înaintarea Puterilor Centrale prin Carpați, dar este depășită după lupte grele, contribuind la ocuparea ulterioară a capitalei.</t>
+          <t>Bătălia de la Târgu Jiu are loc în cadrul apărării Olteniei: trupele române, după lupte grele pe Valea Jiului, încearcă să oprească înaintarea germană, dar orașul cade în mâinile Puterilor Centrale, pregătind marea bătălie de la Neajlov–Argeș și ocuparea Bucureștiului.</t>
         </is>
       </c>
       <c r="R182" s="2" t="inlineStr">
         <is>
-          <t>Depășirea apărării române pe Valea Prahovei</t>
+          <t>Victorie a Puterilor Centrale; căderea Târgu Jiului</t>
         </is>
       </c>
       <c r="S182" s="2" t="inlineStr">
@@ -17755,7 +17755,7 @@
       </c>
       <c r="T182" s="2" t="inlineStr">
         <is>
-          <t>Parte din operația de apărare a trecătorilor din 1916.</t>
+          <t>Parte din a doua bătălie de pe Valea Jiului și din apărarea Olteniei.</t>
         </is>
       </c>
       <c r="U182" s="2" t="inlineStr">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>Bătălia pentru București (1916)</t>
+          <t>Bătălia de pe Neajlov–Argeș (1916)</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
@@ -17782,12 +17782,12 @@
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>1916-11-30</t>
+          <t>1916-11</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>1916-12-03</t>
+          <t>1916-12</t>
         </is>
       </c>
       <c r="F183" s="2" t="n">
@@ -17806,15 +17806,15 @@
       </c>
       <c r="J183" s="2" t="inlineStr">
         <is>
-          <t>București și zona Neajlov–Argeș (județul Ilfov / Dâmbovița)</t>
+          <t>Zona râurilor Neajlov și Argeș, la sud de București</t>
         </is>
       </c>
       <c r="K183" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L183" s="2" t="inlineStr">
         <is>
-          <t>Ilfov / București</t>
+          <t>Giurgiu / Ilfov</t>
         </is>
       </c>
       <c r="M183" s="2" t="inlineStr">
@@ -17823,24 +17823,24 @@
         </is>
       </c>
       <c r="N183" s="2" t="n">
-        <v>44.43</v>
+        <v>44.35</v>
       </c>
       <c r="O183" s="2" t="n">
-        <v>26.1</v>
+        <v>25.75</v>
       </c>
       <c r="P183" s="2" t="inlineStr">
         <is>
-          <t>România vs. Puterile Centrale (Germania, Austro-Ungaria, Bulgaria)</t>
+          <t>România vs. Imperiul German (von Mackensen)</t>
         </is>
       </c>
       <c r="Q183" s="2" t="inlineStr">
         <is>
-          <t>După înfrângerea de la Neajlov–Argeș, germanii și aliații lor înaintează spre capitală. În pofida rezistenței eroice, Bucureștiul este ocupat la 6 decembrie 1916, iar guvernul și armata se retrag în Moldova, marcând prăbușirea frontului de sud.</t>
+          <t>Ultima încercare majoră de a opri înaintarea Puterilor Centrale spre București; după această confruntare, capitala este ocupată.</t>
         </is>
       </c>
       <c r="R183" s="2" t="inlineStr">
         <is>
-          <t>Ocuparea Bucureștiului de către Puterile Centrale</t>
+          <t>Înfrângere românească; ocuparea Bucureștiului</t>
         </is>
       </c>
       <c r="S183" s="2" t="inlineStr">
@@ -17850,12 +17850,12 @@
       </c>
       <c r="T183" s="2" t="inlineStr">
         <is>
-          <t>Parte din operația de apărare a teritoriului Munteniei.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U183" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
+          <t>batalii.csv — sec. XX d.Hr.</t>
         </is>
       </c>
     </row>
@@ -17867,22 +17867,22 @@
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>Operația de la Flămânda</t>
+          <t>Bătălia de pe Valea Jiului (1916)</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Operație / ofensivă</t>
+          <t>Bătălie</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>1916-09-29</t>
+          <t>1916-10</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>1916-10-05</t>
+          <t>1916-11</t>
         </is>
       </c>
       <c r="F184" s="2" t="n">
@@ -17901,7 +17901,7 @@
       </c>
       <c r="J184" s="2" t="inlineStr">
         <is>
-          <t>Zona Flămânda–Oltul și Dunărea de Jos (județul Teleorman / Călărași)</t>
+          <t>Valea Jiului (județele Gorj/Hunedoara)</t>
         </is>
       </c>
       <c r="K184" s="2" t="n">
@@ -17909,33 +17909,33 @@
       </c>
       <c r="L184" s="2" t="inlineStr">
         <is>
-          <t>Teleorman</t>
+          <t>Gorj / Hunedoara</t>
         </is>
       </c>
       <c r="M184" s="2" t="inlineStr">
         <is>
-          <t>Muntenia (sud)</t>
+          <t>Oltenia</t>
         </is>
       </c>
       <c r="N184" s="2" t="n">
-        <v>43.95</v>
+        <v>45.35</v>
       </c>
       <c r="O184" s="2" t="n">
-        <v>25</v>
+        <v>23.15</v>
       </c>
       <c r="P184" s="2" t="inlineStr">
         <is>
-          <t>România (armata a 3-a) vs. Imperiul German și Bulgaria (gruparea Mackensen)</t>
+          <t>România vs. Imperiul German (armata lui Falkenhayn)</t>
         </is>
       </c>
       <c r="Q184" s="2" t="inlineStr">
         <is>
-          <t>Ofensivă românească menită să forțeze Dunărea și să surprindă forțele bulgaro-germane din spate. Operația, nefinalizată și gândită pripit, se soldează cu eșec și este abandonată pe fondul înfrângerii de la Turtucaia și al lipsei de coordonare.</t>
+          <t>Confruntare violentă prin care s-a încercat, fără succes, oprirea înaintării Puterilor Centrale, venite dinspre Transilvania prin Valea Jiului, spre București.</t>
         </is>
       </c>
       <c r="R184" s="2" t="inlineStr">
         <is>
-          <t>Eșecul operației; înfrângerea strategică a României</t>
+          <t>Succes german inițial; depășirea apărării române</t>
         </is>
       </c>
       <c r="S184" s="2" t="inlineStr">
@@ -17945,12 +17945,12 @@
       </c>
       <c r="T184" s="2" t="inlineStr">
         <is>
-          <t>Operație de forțare a Dunării, abandonată din cauza lipsei de coordonare.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U184" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
+          <t>batalii.csv — sec. XX d.Hr.</t>
         </is>
       </c>
     </row>
@@ -17962,7 +17962,7 @@
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>Prima bătălie de la Oituz (1916)</t>
+          <t>Bătălia de pe Valea Prahovei (1916)</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
@@ -17972,12 +17972,12 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>1916-10-12</t>
+          <t>1916-10-09</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
         <is>
-          <t>1916-10-27</t>
+          <t>1916-10-25</t>
         </is>
       </c>
       <c r="F185" s="2" t="n">
@@ -17996,7 +17996,7 @@
       </c>
       <c r="J185" s="2" t="inlineStr">
         <is>
-          <t>Valea Oituzului, Carpații de Curbură (județul Bacău / Covasna)</t>
+          <t>Valea Prahovei, în Carpații Meridionali (județul Prahova)</t>
         </is>
       </c>
       <c r="K185" s="2" t="n">
@@ -18004,19 +18004,19 @@
       </c>
       <c r="L185" s="2" t="inlineStr">
         <is>
-          <t>Bacău</t>
+          <t>Prahova</t>
         </is>
       </c>
       <c r="M185" s="2" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Muntenia</t>
         </is>
       </c>
       <c r="N185" s="2" t="n">
-        <v>46.08</v>
+        <v>45.2</v>
       </c>
       <c r="O185" s="2" t="n">
-        <v>26.35</v>
+        <v>25.7</v>
       </c>
       <c r="P185" s="2" t="inlineStr">
         <is>
@@ -18025,12 +18025,12 @@
       </c>
       <c r="Q185" s="2" t="inlineStr">
         <is>
-          <t>Prima bătălie de la Oituz face parte din apărarea trecătorilor: trupele române opresc înaintarea Puterilor Centrale prin Valea Oituzului, apărând Moldova și împiedicând încercuirea armatei române.</t>
+          <t>Confruntări violente pe valea Prahovei, una dintre principalele căi de acces spre București: armata română încearcă să blocheze înaintarea Puterilor Centrale prin Carpați, dar este depășită după lupte grele, contribuind la ocuparea ulterioară a capitalei.</t>
         </is>
       </c>
       <c r="R185" s="2" t="inlineStr">
         <is>
-          <t>Victorie defensivă a armatei române</t>
+          <t>Depășirea apărării române pe Valea Prahovei</t>
         </is>
       </c>
       <c r="S185" s="2" t="inlineStr">
@@ -18040,7 +18040,7 @@
       </c>
       <c r="T185" s="2" t="inlineStr">
         <is>
-          <t>Urmează a doua bătălie de la Oituz (noiembrie 1916) și cea din 1917.</t>
+          <t>Parte din operația de apărare a trecătorilor din 1916.</t>
         </is>
       </c>
       <c r="U185" s="2" t="inlineStr">
@@ -18057,22 +18057,22 @@
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>Primul Război Mondial — Campania din 1916 (înfrângerea inițială)</t>
+          <t>Bătălia pentru București (1916)</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Campanie / război</t>
+          <t>Bătălie</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>1916-08-27</t>
+          <t>1916-11-30</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>1916-12</t>
+          <t>1916-12-03</t>
         </is>
       </c>
       <c r="F186" s="2" t="n">
@@ -18091,41 +18091,41 @@
       </c>
       <c r="J186" s="2" t="inlineStr">
         <is>
-          <t>Transilvania, Muntenia, Dobrogea, Moldova (capitola de război: Iași)</t>
+          <t>București și zona Neajlov–Argeș (județul Ilfov / Dâmbovița)</t>
         </is>
       </c>
       <c r="K186" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L186" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Ilfov / București</t>
         </is>
       </c>
       <c r="M186" s="2" t="inlineStr">
         <is>
-          <t>România</t>
+          <t>Muntenia</t>
         </is>
       </c>
       <c r="N186" s="2" t="n">
-        <v>46</v>
+        <v>44.43</v>
       </c>
       <c r="O186" s="2" t="n">
-        <v>26</v>
+        <v>26.1</v>
       </c>
       <c r="P186" s="2" t="inlineStr">
         <is>
-          <t>România (Antanta) vs. Puterile Centrale (Imperiul German, Austro-Ungaria, Bulgaria)</t>
+          <t>România vs. Puterile Centrale (Germania, Austro-Ungaria, Bulgaria)</t>
         </is>
       </c>
       <c r="Q186" s="2" t="inlineStr">
         <is>
-          <t>După o ofensivă de scurtă durată în Transilvania, armata română este nevoită să se retragă din cauza atacului combinat al trupelor germane, austro-ungare și bulgare. Sudul țării, inclusiv capitala București, este ocupat de Puterile Centrale; regele, guvernul și armata se retrag în Moldova, Iașiul devenind capitală de război.</t>
+          <t>După înfrângerea de la Neajlov–Argeș, germanii și aliații lor înaintează spre capitală. În pofida rezistenței eroice, Bucureștiul este ocupat la 6 decembrie 1916, iar guvernul și armata se retrag în Moldova, marcând prăbușirea frontului de sud.</t>
         </is>
       </c>
       <c r="R186" s="2" t="inlineStr">
         <is>
-          <t>Ocuparea sudului României; retragerea armatei în Moldova</t>
+          <t>Ocuparea Bucureștiului de către Puterile Centrale</t>
         </is>
       </c>
       <c r="S186" s="2" t="inlineStr">
@@ -18135,12 +18135,12 @@
       </c>
       <c r="T186" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Parte din operația de apărare a teritoriului Munteniei.</t>
         </is>
       </c>
       <c r="U186" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr.</t>
+          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
         </is>
       </c>
     </row>
@@ -18152,29 +18152,29 @@
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Mărășești (1917)</t>
+          <t>Operația de la Flămânda</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>Bătălie</t>
+          <t>Operație / ofensivă</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>1917-08-06</t>
+          <t>1916-09-29</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>1917-09-03</t>
+          <t>1916-10-05</t>
         </is>
       </c>
       <c r="F187" s="2" t="n">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="G187" s="2" t="n">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
@@ -18186,41 +18186,41 @@
       </c>
       <c r="J187" s="2" t="inlineStr">
         <is>
-          <t>Mărășești (județul Vrancea)</t>
+          <t>Zona Flămânda–Oltul și Dunărea de Jos (județul Teleorman / Călărași)</t>
         </is>
       </c>
       <c r="K187" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L187" s="2" t="inlineStr">
         <is>
-          <t>Vrancea</t>
+          <t>Teleorman</t>
         </is>
       </c>
       <c r="M187" s="2" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Muntenia (sud)</t>
         </is>
       </c>
       <c r="N187" s="2" t="n">
-        <v>45.88</v>
+        <v>43.95</v>
       </c>
       <c r="O187" s="2" t="n">
-        <v>27.23</v>
+        <v>25</v>
       </c>
       <c r="P187" s="2" t="inlineStr">
         <is>
-          <t>România vs. Imperiul German (von Mackensen)</t>
+          <t>România (armata a 3-a) vs. Imperiul German și Bulgaria (gruparea Mackensen)</t>
         </is>
       </c>
       <c r="Q187" s="2" t="inlineStr">
         <is>
-          <t>Cea mai mare bătălie de pe frontul românesc: armata română rezistă eroic atacului german, stabilizând frontul sub deviza „Pe aici nu se trece!”.</t>
+          <t>Ofensivă românească menită să forțeze Dunărea și să surprindă forțele bulgaro-germane din spate. Operația, nefinalizată și gândită pripit, se soldează cu eșec și este abandonată pe fondul înfrângerii de la Turtucaia și al lipsei de coordonare.</t>
         </is>
       </c>
       <c r="R187" s="2" t="inlineStr">
         <is>
-          <t>Victorie defensivă românească; stabilizarea frontului</t>
+          <t>Eșecul operației; înfrângerea strategică a României</t>
         </is>
       </c>
       <c r="S187" s="2" t="inlineStr">
@@ -18230,12 +18230,12 @@
       </c>
       <c r="T187" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Operație de forțare a Dunării, abandonată din cauza lipsei de coordonare.</t>
         </is>
       </c>
       <c r="U187" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr.</t>
+          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
         </is>
       </c>
     </row>
@@ -18247,29 +18247,29 @@
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Mărăști (1917)</t>
+          <t>Prima bătălie de la Oituz (1916)</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Bătălie / ofensivă</t>
+          <t>Bătălie</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>1917-07-22</t>
+          <t>1916-10-12</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>1917-08-01</t>
+          <t>1916-10-27</t>
         </is>
       </c>
       <c r="F188" s="2" t="n">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="G188" s="2" t="n">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
@@ -18281,15 +18281,15 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>Mărăști (județul Vrancea)</t>
+          <t>Valea Oituzului, Carpații de Curbură (județul Bacău / Covasna)</t>
         </is>
       </c>
       <c r="K188" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L188" s="2" t="inlineStr">
         <is>
-          <t>Vrancea</t>
+          <t>Bacău</t>
         </is>
       </c>
       <c r="M188" s="2" t="inlineStr">
@@ -18298,24 +18298,24 @@
         </is>
       </c>
       <c r="N188" s="2" t="n">
-        <v>45.83</v>
+        <v>46.08</v>
       </c>
       <c r="O188" s="2" t="n">
-        <v>26.77</v>
+        <v>26.35</v>
       </c>
       <c r="P188" s="2" t="inlineStr">
         <is>
-          <t>România (generalul Alexandru Averescu) vs. Imperiul German și Austro-Ungaria</t>
+          <t>România vs. Imperiul German și Austro-Ungaria</t>
         </is>
       </c>
       <c r="Q188" s="2" t="inlineStr">
         <is>
-          <t>Ofensivă românească reușită, sub conducerea generalului Alexandru Averescu, prin care s-a obținut eliberarea mai multor localități și întărirea moralului armatei române reorganizate.</t>
+          <t>Prima bătălie de la Oituz face parte din apărarea trecătorilor: trupele române opresc înaintarea Puterilor Centrale prin Valea Oituzului, apărând Moldova și împiedicând încercuirea armatei române.</t>
         </is>
       </c>
       <c r="R188" s="2" t="inlineStr">
         <is>
-          <t>Victorie românească; eliberarea unor localități</t>
+          <t>Victorie defensivă a armatei române</t>
         </is>
       </c>
       <c r="S188" s="2" t="inlineStr">
@@ -18325,12 +18325,12 @@
       </c>
       <c r="T188" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Urmează a doua bătălie de la Oituz (noiembrie 1916) și cea din 1917.</t>
         </is>
       </c>
       <c r="U188" s="2" t="inlineStr">
         <is>
-          <t>batalii.csv — sec. XX d.Hr.</t>
+          <t>batalii.csv — sec. XX d.Hr. (completare)</t>
         </is>
       </c>
     </row>
@@ -18342,29 +18342,29 @@
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Oituz (1917)</t>
+          <t>Primul Război Mondial — Campania din 1916 (înfrângerea inițială)</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>Bătălie</t>
+          <t>Campanie / război</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>1917-08-08</t>
+          <t>1916-08-27</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>1917-08-20</t>
+          <t>1916-12</t>
         </is>
       </c>
       <c r="F189" s="2" t="n">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="G189" s="2" t="n">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
@@ -18376,7 +18376,7 @@
       </c>
       <c r="J189" s="2" t="inlineStr">
         <is>
-          <t>Valea Oituzului (județele Bacău/Covasna)</t>
+          <t>Transilvania, Muntenia, Dobrogea, Moldova (capitola de război: Iași)</t>
         </is>
       </c>
       <c r="K189" s="2" t="n">
@@ -18384,33 +18384,33 @@
       </c>
       <c r="L189" s="2" t="inlineStr">
         <is>
-          <t>Bacău / Covasna</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M189" s="2" t="inlineStr">
         <is>
-          <t>Moldova / Transilvania</t>
+          <t>România</t>
         </is>
       </c>
       <c r="N189" s="2" t="n">
-        <v>46.1</v>
+        <v>46</v>
       </c>
       <c r="O189" s="2" t="n">
-        <v>26.43</v>
+        <v>26</v>
       </c>
       <c r="P189" s="2" t="inlineStr">
         <is>
-          <t>România vs. Imperiul German și Austro-Ungaria</t>
+          <t>România (Antanta) vs. Puterile Centrale (Imperiul German, Austro-Ungaria, Bulgaria)</t>
         </is>
       </c>
       <c r="Q189" s="2" t="inlineStr">
         <is>
-          <t>Desfășurată în paralel cu bătălia de la Mărășești, trupele române blochează încercarea inamicului de a pătrunde în valea Trotușului, în inima Moldovei.</t>
+          <t>După o ofensivă de scurtă durată în Transilvania, armata română este nevoită să se retragă din cauza atacului combinat al trupelor germane, austro-ungare și bulgare. Sudul țării, inclusiv capitala București, este ocupat de Puterile Centrale; regele, guvernul și armata se retrag în Moldova, Iașiul devenind capitală de război.</t>
         </is>
       </c>
       <c r="R189" s="2" t="inlineStr">
         <is>
-          <t>Victorie defensivă românească</t>
+          <t>Ocuparea sudului României; retragerea armatei în Moldova</t>
         </is>
       </c>
       <c r="S189" s="2" t="inlineStr">
@@ -18437,29 +18437,29 @@
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>Al Doilea Război Mondial — Operațiunea Tidal Wave (bombardarea Ploieștiului)</t>
+          <t>Bătălia de la Mărășești (1917)</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Bombardament aerian</t>
+          <t>Bătălie</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>1943-08-01</t>
+          <t>1917-08-06</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>1943-08-01</t>
+          <t>1917-09-03</t>
         </is>
       </c>
       <c r="F190" s="2" t="n">
-        <v>1943</v>
+        <v>1917</v>
       </c>
       <c r="G190" s="2" t="n">
-        <v>1943</v>
+        <v>1917</v>
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
@@ -18471,7 +18471,7 @@
       </c>
       <c r="J190" s="2" t="inlineStr">
         <is>
-          <t>Ploiești (județul Prahova)</t>
+          <t>Mărășești (județul Vrancea)</t>
         </is>
       </c>
       <c r="K190" s="2" t="n">
@@ -18479,33 +18479,33 @@
       </c>
       <c r="L190" s="2" t="inlineStr">
         <is>
-          <t>Prahova</t>
+          <t>Vrancea</t>
         </is>
       </c>
       <c r="M190" s="2" t="inlineStr">
         <is>
-          <t>Muntenia</t>
+          <t>Moldova</t>
         </is>
       </c>
       <c r="N190" s="2" t="n">
-        <v>44.94</v>
+        <v>45.88</v>
       </c>
       <c r="O190" s="2" t="n">
-        <v>26.02</v>
+        <v>27.23</v>
       </c>
       <c r="P190" s="2" t="inlineStr">
         <is>
-          <t>SUA (USAAF) vs. România (apărarea antiaeriană) și Germania Nazistă (apărarea rafinăriilor)</t>
+          <t>România vs. Imperiul German (von Mackensen)</t>
         </is>
       </c>
       <c r="Q190" s="2" t="inlineStr">
         <is>
-          <t>Atac aerian masiv al aviației americane (USAAF) asupra rafinăriilor de petrol de la Ploiești — una dintre cele mai sângeroase și costisitoare misiuni aeriene pentru americani din întreg războiul.</t>
+          <t>Cea mai mare bătălie de pe frontul românesc: armata română rezistă eroic atacului german, stabilizând frontul sub deviza „Pe aici nu se trece!”.</t>
         </is>
       </c>
       <c r="R190" s="2" t="inlineStr">
         <is>
-          <t>Distrugeri parțiale ale rafinăriilor, cu pierderi aeriene americane mari</t>
+          <t>Victorie defensivă românească; stabilizarea frontului</t>
         </is>
       </c>
       <c r="S190" s="2" t="inlineStr">
@@ -18532,29 +18532,29 @@
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>Bombardamentele aliate asupra României (1943–1944)</t>
+          <t>Bătălia de la Mărăști (1917)</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>Bombardamente aeriene</t>
+          <t>Bătălie / ofensivă</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>1917-07-22</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1917-08-01</t>
         </is>
       </c>
       <c r="F191" s="2" t="n">
-        <v>1943</v>
+        <v>1917</v>
       </c>
       <c r="G191" s="2" t="n">
-        <v>1944</v>
+        <v>1917</v>
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
@@ -18566,41 +18566,41 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>București, Ploiești, Turnu Severin, Brașov</t>
+          <t>Mărăști (județul Vrancea)</t>
         </is>
       </c>
       <c r="K191" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L191" s="2" t="inlineStr">
         <is>
-          <t>Ilfov / Prahova / Mehedinți / Brașov</t>
+          <t>Vrancea</t>
         </is>
       </c>
       <c r="M191" s="2" t="inlineStr">
         <is>
-          <t>România</t>
+          <t>Moldova</t>
         </is>
       </c>
       <c r="N191" s="2" t="n">
-        <v>44.8</v>
+        <v>45.83</v>
       </c>
       <c r="O191" s="2" t="n">
-        <v>25.4</v>
+        <v>26.77</v>
       </c>
       <c r="P191" s="2" t="inlineStr">
         <is>
-          <t>Aliații (SUA — USAAF, Regatul Unit — RAF) vs. România și Germania Nazistă</t>
+          <t>România (generalul Alexandru Averescu) vs. Imperiul German și Austro-Ungaria</t>
         </is>
       </c>
       <c r="Q191" s="2" t="inlineStr">
         <is>
-          <t>Înainte de intrarea trupelor terestre, România este ținta unor intense atacuri aeriene americane și britanice, având ca scop distrugerea infrastructurii petroliere și feroviare. Orașe precum București (inclusiv atacul devastator din 4 aprilie 1944 asupra Gării de Nord), Ploiești, Turnu Severin și Brașov sunt bombardate sistematic.</t>
+          <t>Ofensivă românească reușită, sub conducerea generalului Alexandru Averescu, prin care s-a obținut eliberarea mai multor localități și întărirea moralului armatei române reorganizate.</t>
         </is>
       </c>
       <c r="R191" s="2" t="inlineStr">
         <is>
-          <t>Distrugeri ale infrastructurii; victime civile numeroase</t>
+          <t>Victorie românească; eliberarea unor localități</t>
         </is>
       </c>
       <c r="S191" s="2" t="inlineStr">
@@ -18627,29 +18627,29 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>A Doua Ofensivă Iași–Chișinău (20–29 august 1944)</t>
+          <t>Bătălia de la Oituz (1917)</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Ofensivă strategică</t>
+          <t>Bătălie</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>1944-08-20</t>
+          <t>1917-08-08</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>1944-08-29</t>
+          <t>1917-08-20</t>
         </is>
       </c>
       <c r="F192" s="2" t="n">
-        <v>1944</v>
+        <v>1917</v>
       </c>
       <c r="G192" s="2" t="n">
-        <v>1944</v>
+        <v>1917</v>
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
@@ -18661,7 +18661,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>Moldova: Iași, Chișinău, frontul germano-român</t>
+          <t>Valea Oituzului (județele Bacău/Covasna)</t>
         </is>
       </c>
       <c r="K192" s="2" t="n">
@@ -18669,33 +18669,33 @@
       </c>
       <c r="L192" s="2" t="inlineStr">
         <is>
-          <t>Iași</t>
+          <t>Bacău / Covasna</t>
         </is>
       </c>
       <c r="M192" s="2" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Moldova / Transilvania</t>
         </is>
       </c>
       <c r="N192" s="2" t="n">
-        <v>47.1</v>
+        <v>46.1</v>
       </c>
       <c r="O192" s="2" t="n">
-        <v>27.5</v>
+        <v>26.43</v>
       </c>
       <c r="P192" s="2" t="inlineStr">
         <is>
-          <t>URSS (Armata Roșie) vs. România și Germania Nazistă</t>
+          <t>România vs. Imperiul German și Austro-Ungaria</t>
         </is>
       </c>
       <c r="Q192" s="2" t="inlineStr">
         <is>
-          <t>Operațiune strategică sovietică masivă care duce la prăbușirea completă a frontului germano-român din Moldova: Armata Roșie sparge rapid liniile defensive de la Iași și Chișinău. Prăbușirea militară accelerează lovitura de stat de la București din 23 august 1944.</t>
+          <t>Desfășurată în paralel cu bătălia de la Mărășești, trupele române blochează încercarea inamicului de a pătrunde în valea Trotușului, în inima Moldovei.</t>
         </is>
       </c>
       <c r="R192" s="2" t="inlineStr">
         <is>
-          <t>Prăbușirea frontului; lovitura de stat din 23 august 1944</t>
+          <t>Victorie defensivă românească</t>
         </is>
       </c>
       <c r="S192" s="2" t="inlineStr">
@@ -18722,29 +18722,29 @@
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Păuliș (1944)</t>
+          <t>Al Doilea Război Mondial — Operațiunea Tidal Wave (bombardarea Ploieștiului)</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Bătălie defensivă</t>
+          <t>Bombardament aerian</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>1944-09-14</t>
+          <t>1943-08-01</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>1944-09-19</t>
+          <t>1943-08-01</t>
         </is>
       </c>
       <c r="F193" s="2" t="n">
-        <v>1944</v>
+        <v>1943</v>
       </c>
       <c r="G193" s="2" t="n">
-        <v>1944</v>
+        <v>1943</v>
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
@@ -18756,7 +18756,7 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>Păuliș (județul Arad)</t>
+          <t>Ploiești (județul Prahova)</t>
         </is>
       </c>
       <c r="K193" s="2" t="n">
@@ -18764,33 +18764,33 @@
       </c>
       <c r="L193" s="2" t="inlineStr">
         <is>
-          <t>Arad</t>
+          <t>Prahova</t>
         </is>
       </c>
       <c r="M193" s="2" t="inlineStr">
         <is>
-          <t>Banat</t>
+          <t>Muntenia</t>
         </is>
       </c>
       <c r="N193" s="2" t="n">
-        <v>46.12</v>
+        <v>44.94</v>
       </c>
       <c r="O193" s="2" t="n">
-        <v>21.59</v>
+        <v>26.02</v>
       </c>
       <c r="P193" s="2" t="inlineStr">
         <is>
-          <t>România (elevii Școlii de Subofițeri de Rezervă de la Radna) vs. Ungaria (armata horthystă)</t>
+          <t>SUA (USAAF) vs. România (apărarea antiaeriană) și Germania Nazistă (apărarea rafinăriilor)</t>
         </is>
       </c>
       <c r="Q193" s="2" t="inlineStr">
         <is>
-          <t>Elevii școlii de subofițeri de rezervă de la Radna opresc o ofensivă puternică a trupelor ungare, într-una dintre cele mai eroice confruntări defensive ale campaniei din vestul României.</t>
+          <t>Atac aerian masiv al aviației americane (USAAF) asupra rafinăriilor de petrol de la Ploiești — una dintre cele mai sângeroase și costisitoare misiuni aeriene pentru americani din întreg războiul.</t>
         </is>
       </c>
       <c r="R193" s="2" t="inlineStr">
         <is>
-          <t>Victorie defensivă românească împotriva forțelor superioare</t>
+          <t>Distrugeri parțiale ale rafinăriilor, cu pierderi aeriene americane mari</t>
         </is>
       </c>
       <c r="S193" s="2" t="inlineStr">
@@ -18817,26 +18817,26 @@
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>Bătălia de la Turda (1944)</t>
+          <t>Bombardamentele aliate asupra României (1943–1944)</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Bătălie de blindate</t>
+          <t>Bombardamente aeriene</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>1944-09</t>
+          <t>1943</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>1944-10</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="F194" s="2" t="n">
-        <v>1944</v>
+        <v>1943</v>
       </c>
       <c r="G194" s="2" t="n">
         <v>1944</v>
@@ -18851,41 +18851,41 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>Turda (județul Cluj)</t>
+          <t>București, Ploiești, Turnu Severin, Brașov</t>
         </is>
       </c>
       <c r="K194" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
-          <t>Cluj</t>
+          <t>Ilfov / Prahova / Mehedinți / Brașov</t>
         </is>
       </c>
       <c r="M194" s="2" t="inlineStr">
         <is>
-          <t>Transilvania</t>
+          <t>România</t>
         </is>
       </c>
       <c r="N194" s="2" t="n">
-        <v>46.57</v>
+        <v>44.8</v>
       </c>
       <c r="O194" s="2" t="n">
-        <v>23.78</v>
+        <v>25.4</v>
       </c>
       <c r="P194" s="2" t="inlineStr">
         <is>
-          <t>România și URSS vs. Germania Nazistă și Ungaria</t>
+          <t>Aliații (SUA — USAAF, Regatul Unit — RAF) vs. România și Germania Nazistă</t>
         </is>
       </c>
       <c r="Q194" s="2" t="inlineStr">
         <is>
-          <t>Una dintre cele mai mari și mai grele bătălii de blindate de pe teritoriul actual al României: trupele ungaro-germane opun o rezistență dârză în fața forțelor româno-sovietice, în cadrul campaniei de eliberare a Transilvaniei de Nord.</t>
+          <t>Înainte de intrarea trupelor terestre, România este ținta unor intense atacuri aeriene americane și britanice, având ca scop distrugerea infrastructurii petroliere și feroviare. Orașe precum București (inclusiv atacul devastator din 4 aprilie 1944 asupra Gării de Nord), Ploiești, Turnu Severin și Brașov sunt bombardate sistematic.</t>
         </is>
       </c>
       <c r="R194" s="2" t="inlineStr">
         <is>
-          <t>Cucerirea Turdei de către forțele româno-sovietice</t>
+          <t>Distrugeri ale infrastructurii; victime civile numeroase</t>
         </is>
       </c>
       <c r="S194" s="2" t="inlineStr">
@@ -18912,22 +18912,22 @@
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>Bătălia pentru București (august–septembrie 1944)</t>
+          <t>A Doua Ofensivă Iași–Chișinău (20–29 august 1944)</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Bătălie urbană</t>
+          <t>Ofensivă strategică</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>1944-08-24</t>
+          <t>1944-08-20</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
-          <t>1944-09</t>
+          <t>1944-08-29</t>
         </is>
       </c>
       <c r="F195" s="2" t="n">
@@ -18946,7 +18946,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>București</t>
+          <t>Moldova: Iași, Chișinău, frontul germano-român</t>
         </is>
       </c>
       <c r="K195" s="2" t="n">
@@ -18954,33 +18954,33 @@
       </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
-          <t>Ilfov</t>
+          <t>Iași</t>
         </is>
       </c>
       <c r="M195" s="2" t="inlineStr">
         <is>
-          <t>Muntenia</t>
+          <t>Moldova</t>
         </is>
       </c>
       <c r="N195" s="2" t="n">
-        <v>44.43</v>
+        <v>47.1</v>
       </c>
       <c r="O195" s="2" t="n">
-        <v>26.1</v>
+        <v>27.5</v>
       </c>
       <c r="P195" s="2" t="inlineStr">
         <is>
-          <t>România (armata, după 23 august) vs. Germania Nazistă</t>
+          <t>URSS (Armata Roșie) vs. România și Germania Nazistă</t>
         </is>
       </c>
       <c r="Q195" s="2" t="inlineStr">
         <is>
-          <t>După actul de la 23 august 1944, teritoriul României devine teatrul unor lupte intense între foștii aliați. Trupele române resping atacurile germane care încercau să ocupe Capitala și să instaureze un regim marionetă; până la sosirea sovieticilor, Bucureștiul este deja eliberat de armata română.</t>
+          <t>Operațiune strategică sovietică masivă care duce la prăbușirea completă a frontului germano-român din Moldova: Armata Roșie sparge rapid liniile defensive de la Iași și Chișinău. Prăbușirea militară accelerează lovitura de stat de la București din 23 august 1944.</t>
         </is>
       </c>
       <c r="R195" s="2" t="inlineStr">
         <is>
-          <t>Eliberarea Bucureștiului de către armata română</t>
+          <t>Prăbușirea frontului; lovitura de stat din 23 august 1944</t>
         </is>
       </c>
       <c r="S195" s="2" t="inlineStr">
@@ -19007,22 +19007,22 @@
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>Eliberarea Careiului și Satu Mare (25 octombrie 1944)</t>
+          <t>Bătălia de la Păuliș (1944)</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Ofensivă / eliberare</t>
+          <t>Bătălie defensivă</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>1944-10</t>
+          <t>1944-09-14</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>1944-10-25</t>
+          <t>1944-09-19</t>
         </is>
       </c>
       <c r="F196" s="2" t="n">
@@ -19041,41 +19041,41 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>Carei și Satu Mare</t>
+          <t>Păuliș (județul Arad)</t>
         </is>
       </c>
       <c r="K196" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
-          <t>Satu Mare</t>
+          <t>Arad</t>
         </is>
       </c>
       <c r="M196" s="2" t="inlineStr">
         <is>
-          <t>Transilvania (nord-vest)</t>
+          <t>Banat</t>
         </is>
       </c>
       <c r="N196" s="2" t="n">
-        <v>47.74</v>
+        <v>46.12</v>
       </c>
       <c r="O196" s="2" t="n">
-        <v>22.68</v>
+        <v>21.59</v>
       </c>
       <c r="P196" s="2" t="inlineStr">
         <is>
-          <t>România și URSS vs. Germania Nazistă și Ungaria</t>
+          <t>România (elevii Școlii de Subofițeri de Rezervă de la Radna) vs. Ungaria (armata horthystă)</t>
         </is>
       </c>
       <c r="Q196" s="2" t="inlineStr">
         <is>
-          <t>Armata română, acționând împreună cu Armata Roșie, eliberează în 25 octombrie 1944 orașele Carei și Satu Mare, încheind eliberarea întregului teritoriu actual al României de sub ocupația trupelor Axei.</t>
+          <t>Elevii școlii de subofițeri de rezervă de la Radna opresc o ofensivă puternică a trupelor ungare, într-una dintre cele mai eroice confruntări defensive ale campaniei din vestul României.</t>
         </is>
       </c>
       <c r="R196" s="2" t="inlineStr">
         <is>
-          <t>Eliberarea completă a teritoriului României (25 oct. 1944)</t>
+          <t>Victorie defensivă românească împotriva forțelor superioare</t>
         </is>
       </c>
       <c r="S196" s="2" t="inlineStr">
@@ -19102,22 +19102,22 @@
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>Luptele de pe linia Dunării și din Dobrogea (1944)</t>
+          <t>Bătălia de la Turda (1944)</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Lupte de retragere / blocare</t>
+          <t>Bătălie de blindate</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>1944-08</t>
+          <t>1944-09</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>1944-09</t>
+          <t>1944-10</t>
         </is>
       </c>
       <c r="F197" s="2" t="n">
@@ -19136,41 +19136,41 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>Dunărea de Jos și Dobrogea</t>
+          <t>Turda (județul Cluj)</t>
         </is>
       </c>
       <c r="K197" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L197" s="2" t="inlineStr">
         <is>
-          <t>Constanța / Tulcea / Călărași</t>
+          <t>Cluj</t>
         </is>
       </c>
       <c r="M197" s="2" t="inlineStr">
         <is>
-          <t>Dobrogea</t>
+          <t>Transilvania</t>
         </is>
       </c>
       <c r="N197" s="2" t="n">
-        <v>44.4</v>
+        <v>46.57</v>
       </c>
       <c r="O197" s="2" t="n">
-        <v>28</v>
+        <v>23.78</v>
       </c>
       <c r="P197" s="2" t="inlineStr">
         <is>
-          <t>România și URSS vs. Germania Nazistă</t>
+          <t>România și URSS vs. Germania Nazistă și Ungaria</t>
         </is>
       </c>
       <c r="Q197" s="2" t="inlineStr">
         <is>
-          <t>Confruntări pentru blocarea retragerii trupelor germane din Balcani, desfășurate pe linia Dunării și în Dobrogea, ca parte a luptelor de după 23 august 1944.</t>
+          <t>Una dintre cele mai mari și mai grele bătălii de blindate de pe teritoriul actual al României: trupele ungaro-germane opun o rezistență dârză în fața forțelor româno-sovietice, în cadrul campaniei de eliberare a Transilvaniei de Nord.</t>
         </is>
       </c>
       <c r="R197" s="2" t="inlineStr">
         <is>
-          <t>Blocarea și capturarea unor forțe germane care se retrăgeau</t>
+          <t>Cucerirea Turdei de către forțele româno-sovietice</t>
         </is>
       </c>
       <c r="S197" s="2" t="inlineStr">
@@ -19197,22 +19197,22 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>Ofensiva Uman–Botoșani (1944)</t>
+          <t>Bătălia pentru București (august–septembrie 1944)</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Ofensivă</t>
+          <t>Bătălie urbană</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>1944-03</t>
+          <t>1944-08-24</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>1944-04</t>
+          <t>1944-09</t>
         </is>
       </c>
       <c r="F198" s="2" t="n">
@@ -19231,7 +19231,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>Nordul Moldovei: Botoșani, Dorohoi, Suceava</t>
+          <t>București</t>
         </is>
       </c>
       <c r="K198" s="2" t="n">
@@ -19239,33 +19239,33 @@
       </c>
       <c r="L198" s="2" t="inlineStr">
         <is>
-          <t>Botoșani / Suceava</t>
+          <t>Ilfov</t>
         </is>
       </c>
       <c r="M198" s="2" t="inlineStr">
         <is>
-          <t>Moldova</t>
+          <t>Muntenia</t>
         </is>
       </c>
       <c r="N198" s="2" t="n">
-        <v>47.8</v>
+        <v>44.43</v>
       </c>
       <c r="O198" s="2" t="n">
-        <v>26.5</v>
+        <v>26.1</v>
       </c>
       <c r="P198" s="2" t="inlineStr">
         <is>
-          <t>URSS (Armata Roșie) vs. România și Germania Nazistă</t>
+          <t>România (armata, după 23 august) vs. Germania Nazistă</t>
         </is>
       </c>
       <c r="Q198" s="2" t="inlineStr">
         <is>
-          <t>Ofensiva marchează intrarea trupelor sovietice pe teritoriul României: Frontul de Est ajunge în nordul Moldovei, iar sovieticii ocupă orașe precum Botoșani, Dorohoi și Suceava, stabilind linia frontului în nordul țării.</t>
+          <t>După actul de la 23 august 1944, teritoriul României devine teatrul unor lupte intense între foștii aliați. Trupele române resping atacurile germane care încercau să ocupe Capitala și să instaureze un regim marionetă; până la sosirea sovieticilor, Bucureștiul este deja eliberat de armata română.</t>
         </is>
       </c>
       <c r="R198" s="2" t="inlineStr">
         <is>
-          <t>Ocuparea nordului Moldovei de către Armata Roșie</t>
+          <t>Eliberarea Bucureștiului de către armata română</t>
         </is>
       </c>
       <c r="S198" s="2" t="inlineStr">
@@ -19292,22 +19292,22 @@
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>Prima Ofensivă Iași–Chișinău (1944) și bătălia de la Târgu Frumos</t>
+          <t>Eliberarea Careiului și Satu Mare (25 octombrie 1944)</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Ofensivă / bătălie de blindate</t>
+          <t>Ofensivă / eliberare</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>1944-04-08</t>
+          <t>1944-10</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>1944-06-06</t>
+          <t>1944-10-25</t>
         </is>
       </c>
       <c r="F199" s="2" t="n">
@@ -19326,61 +19326,346 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
+          <t>Carei și Satu Mare</t>
+        </is>
+      </c>
+      <c r="K199" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L199" s="2" t="inlineStr">
+        <is>
+          <t>Satu Mare</t>
+        </is>
+      </c>
+      <c r="M199" s="2" t="inlineStr">
+        <is>
+          <t>Transilvania (nord-vest)</t>
+        </is>
+      </c>
+      <c r="N199" s="2" t="n">
+        <v>47.74</v>
+      </c>
+      <c r="O199" s="2" t="n">
+        <v>22.68</v>
+      </c>
+      <c r="P199" s="2" t="inlineStr">
+        <is>
+          <t>România și URSS vs. Germania Nazistă și Ungaria</t>
+        </is>
+      </c>
+      <c r="Q199" s="2" t="inlineStr">
+        <is>
+          <t>Armata română, acționând împreună cu Armata Roșie, eliberează în 25 octombrie 1944 orașele Carei și Satu Mare, încheind eliberarea întregului teritoriu actual al României de sub ocupația trupelor Axei.</t>
+        </is>
+      </c>
+      <c r="R199" s="2" t="inlineStr">
+        <is>
+          <t>Eliberarea completă a teritoriului României (25 oct. 1944)</t>
+        </is>
+      </c>
+      <c r="S199" s="2" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
+      <c r="T199" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U199" s="2" t="inlineStr">
+        <is>
+          <t>batalii.csv — sec. XX d.Hr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>RM-199</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>Luptele de pe linia Dunării și din Dobrogea (1944)</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Lupte de retragere / blocare</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>1944-08</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>1944-09</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="n">
+        <v>1944</v>
+      </c>
+      <c r="G200" s="2" t="n">
+        <v>1944</v>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>sec. XX d.Hr.</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>Dunărea de Jos și Dobrogea</t>
+        </is>
+      </c>
+      <c r="K200" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L200" s="2" t="inlineStr">
+        <is>
+          <t>Constanța / Tulcea / Călărași</t>
+        </is>
+      </c>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>Dobrogea</t>
+        </is>
+      </c>
+      <c r="N200" s="2" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="O200" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="P200" s="2" t="inlineStr">
+        <is>
+          <t>România și URSS vs. Germania Nazistă</t>
+        </is>
+      </c>
+      <c r="Q200" s="2" t="inlineStr">
+        <is>
+          <t>Confruntări pentru blocarea retragerii trupelor germane din Balcani, desfășurate pe linia Dunării și în Dobrogea, ca parte a luptelor de după 23 august 1944.</t>
+        </is>
+      </c>
+      <c r="R200" s="2" t="inlineStr">
+        <is>
+          <t>Blocarea și capturarea unor forțe germane care se retrăgeau</t>
+        </is>
+      </c>
+      <c r="S200" s="2" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
+      <c r="T200" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U200" s="2" t="inlineStr">
+        <is>
+          <t>batalii.csv — sec. XX d.Hr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>RM-200</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>Ofensiva Uman–Botoșani (1944)</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>Ofensivă</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>1944-03</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>1944-04</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="n">
+        <v>1944</v>
+      </c>
+      <c r="G201" s="2" t="n">
+        <v>1944</v>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>sec. XX d.Hr.</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>Nordul Moldovei: Botoșani, Dorohoi, Suceava</t>
+        </is>
+      </c>
+      <c r="K201" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L201" s="2" t="inlineStr">
+        <is>
+          <t>Botoșani / Suceava</t>
+        </is>
+      </c>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t>Moldova</t>
+        </is>
+      </c>
+      <c r="N201" s="2" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="O201" s="2" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="P201" s="2" t="inlineStr">
+        <is>
+          <t>URSS (Armata Roșie) vs. România și Germania Nazistă</t>
+        </is>
+      </c>
+      <c r="Q201" s="2" t="inlineStr">
+        <is>
+          <t>Ofensiva marchează intrarea trupelor sovietice pe teritoriul României: Frontul de Est ajunge în nordul Moldovei, iar sovieticii ocupă orașe precum Botoșani, Dorohoi și Suceava, stabilind linia frontului în nordul țării.</t>
+        </is>
+      </c>
+      <c r="R201" s="2" t="inlineStr">
+        <is>
+          <t>Ocuparea nordului Moldovei de către Armata Roșie</t>
+        </is>
+      </c>
+      <c r="S201" s="2" t="inlineStr">
+        <is>
+          <t>Da</t>
+        </is>
+      </c>
+      <c r="T201" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U201" s="2" t="inlineStr">
+        <is>
+          <t>batalii.csv — sec. XX d.Hr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>RM-201</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>Prima Ofensivă Iași–Chișinău (1944) și bătălia de la Târgu Frumos</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Ofensivă / bătălie de blindate</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>1944-04-08</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>1944-06-06</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="n">
+        <v>1944</v>
+      </c>
+      <c r="G202" s="2" t="n">
+        <v>1944</v>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>sec. XX d.Hr.</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
           <t>Moldova: Târgu Frumos, valea Siretului, Iași–Chișinău</t>
         </is>
       </c>
-      <c r="K199" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L199" s="2" t="inlineStr">
+      <c r="K202" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L202" s="2" t="inlineStr">
         <is>
           <t>Iași / Neamț</t>
         </is>
       </c>
-      <c r="M199" s="2" t="inlineStr">
+      <c r="M202" s="2" t="inlineStr">
         <is>
           <t>Moldova</t>
         </is>
       </c>
-      <c r="N199" s="2" t="n">
+      <c r="N202" s="2" t="n">
         <v>47.21</v>
       </c>
-      <c r="O199" s="2" t="n">
+      <c r="O202" s="2" t="n">
         <v>26.99</v>
       </c>
-      <c r="P199" s="2" t="inlineStr">
+      <c r="P202" s="2" t="inlineStr">
         <is>
           <t>URSS (Armata Roșie) vs. România și Germania Nazistă (generalul Hasso von Manteuffel)</t>
         </is>
       </c>
-      <c r="Q199" s="2" t="inlineStr">
+      <c r="Q202" s="2" t="inlineStr">
         <is>
           <t>Serie de lupte violente de uzură între trupele germano-române și cele sovietice. Bătălia de la Târgu Frumos este o confruntare de blindate de mare amploare, unde trupele germane și cele române reușesc temporar să oprească avansul tancurilor sovietice.</t>
         </is>
       </c>
-      <c r="R199" s="2" t="inlineStr">
+      <c r="R202" s="2" t="inlineStr">
         <is>
           <t>Stoparea temporară a ofensivei sovietice</t>
         </is>
       </c>
-      <c r="S199" s="2" t="inlineStr">
+      <c r="S202" s="2" t="inlineStr">
         <is>
           <t>Da</t>
         </is>
       </c>
-      <c r="T199" s="2" t="inlineStr">
+      <c r="T202" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="U199" s="2" t="inlineStr">
+      <c r="U202" s="2" t="inlineStr">
         <is>
           <t>batalii.csv — sec. XX d.Hr.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U199"/>
+  <autoFilter ref="A1:U202"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19417,7 +19702,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3">
@@ -19427,7 +19712,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4">
@@ -19499,7 +19784,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -19791,7 +20076,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42">
@@ -19827,7 +20112,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Invazie</t>
+          <t>Asediu</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -19837,7 +20122,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Bătălie (context regional)</t>
+          <t>Invazie</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -19847,7 +20132,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Campanii / expediții</t>
+          <t>Bătălie (context regional)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -19857,17 +20142,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Conflicte de frontieră</t>
+          <t>Campanii / expediții</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Incursiuni de jaf</t>
+          <t>Conflicte de frontieră</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -19877,7 +20162,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Campanie</t>
+          <t>Incursiuni de jaf</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -19887,7 +20172,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Războaie / campanii</t>
+          <t>Campanie</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -19897,7 +20182,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Campanie / cucerire</t>
+          <t>Războaie / campanii</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -19907,7 +20192,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Război / cucerire</t>
+          <t>Campanie / cucerire</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -19917,7 +20202,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Asediu</t>
+          <t>Război / cucerire</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -20829,17 +21114,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Transilvania</t>
+          <t>Dobrogea</t>
         </is>
       </c>
       <c r="B146" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Dobrogea</t>
+          <t>Transilvania</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -20863,7 +21148,7 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="150">
@@ -20899,17 +21184,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Moldova / Muntenia</t>
+          <t>Banat</t>
         </is>
       </c>
       <c r="B153" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Banat</t>
+          <t>Moldova / Muntenia</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -20979,7 +21264,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Oltenia</t>
+          <t>Crișana</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -20989,7 +21274,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Bulgaria (în afara actualelor granițe)</t>
+          <t>Oltenia</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -20999,17 +21284,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Muntenia / Oltenia</t>
+          <t>Bulgaria (în afara actualelor granițe)</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Transilvania / Oltenia</t>
+          <t>Muntenia / Oltenia</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -21019,7 +21304,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Banat / Crișana / Transilvania (vest)</t>
+          <t>Transilvania / Oltenia</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -21029,7 +21314,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Oltenia / Muntenia</t>
+          <t>Banat / Crișana / Transilvania (vest)</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -21039,7 +21324,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Muntenia / Oltenia / Dobrogea</t>
+          <t>Oltenia / Muntenia</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -21049,7 +21334,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Transilvania / Banat</t>
+          <t>Muntenia / Oltenia / Dobrogea</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -21059,7 +21344,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Transilvania / Banat / Crișana</t>
+          <t>Transilvania / Banat</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -21069,7 +21354,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Crișana</t>
+          <t>Transilvania / Banat / Crișana</t>
         </is>
       </c>
       <c r="B170" t="n">

</xml_diff>